<commit_message>
Atualizando Registros_2026.xlsx via script Python
</commit_message>
<xml_diff>
--- a/Arquivos_Origem/Registros_2026.xlsx
+++ b/Arquivos_Origem/Registros_2026.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Transações" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Transações" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Transações'!$A$1:$J$1630</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Transações'!$A$1:$J$1632</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J1630"/>
+  <dimension ref="A1:J1632"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -540,20 +540,20 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Combustível para a HILUX</t>
+          <t>Ajuda aos necessitados</t>
         </is>
       </c>
       <c r="C3" s="3" t="n">
-        <v>-230.4</v>
+        <v>-60</v>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Combustível</t>
+          <t>Doações e Ajudas</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Cartão BB VISA</t>
+          <t>Conta BB</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
@@ -563,12 +563,12 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>TRANSPORTE</t>
+          <t>DOAÇÕES</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>Despesas com Combustível</t>
+          <t>Despesas com doações</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
@@ -583,20 +583,20 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Alimentos e Materiais de limpeza</t>
+          <t>Serviço Apartamento 42 - São Paulo (P 2)</t>
         </is>
       </c>
       <c r="C4" s="3" t="n">
-        <v>-924.88</v>
+        <v>-2801</v>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Supermercado</t>
+          <t>OUTRAS DESPESAS</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Cartão BB VISA</t>
+          <t>Conta BB</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
@@ -606,12 +606,12 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>ALIMENTAÇÃO E LIMPEZA</t>
+          <t>OUTRAS DESPESAS</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>Despesas com alimentação e limpeza</t>
+          <t>Outras Despesas</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
@@ -626,20 +626,20 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Apt. Aju. - Energia Elétrica</t>
+          <t>Alimentos e Materiais de limpeza</t>
         </is>
       </c>
       <c r="C5" s="3" t="n">
-        <v>-214.23</v>
+        <v>-924.88</v>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Energia Elétrica</t>
+          <t>Supermercado</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Conta BB</t>
+          <t>Cartão BB VISA</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
@@ -649,17 +649,12 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>IMÓVEIS</t>
-        </is>
-      </c>
-      <c r="H5" t="inlineStr">
-        <is>
-          <t>Contas da casa</t>
+          <t>ALIMENTAÇÃO E LIMPEZA</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>Despesas com imóveis</t>
+          <t>Despesas com alimentação e limpeza</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
@@ -674,15 +669,15 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Ajuda aos necessitados</t>
+          <t>Apt. Aju. - Energia Elétrica</t>
         </is>
       </c>
       <c r="C6" s="3" t="n">
-        <v>-60</v>
+        <v>-214.23</v>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Doações e Ajudas</t>
+          <t>Energia Elétrica</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
@@ -697,12 +692,17 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>DOAÇÕES</t>
+          <t>IMÓVEIS</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>Contas da casa</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>Despesas com doações</t>
+          <t>Despesas com imóveis</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
@@ -717,20 +717,20 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Serviço Apartamento 42 - São Paulo (P 2)</t>
+          <t>Combustível para a HILUX</t>
         </is>
       </c>
       <c r="C7" s="3" t="n">
-        <v>-2801</v>
+        <v>-230.4</v>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>OUTRAS DESPESAS</t>
+          <t>Combustível</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Conta BB</t>
+          <t>Cartão BB VISA</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
@@ -740,12 +740,12 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>OUTRAS DESPESAS</t>
+          <t>TRANSPORTE</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>Outras Despesas</t>
+          <t>Despesas com Combustível</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
@@ -851,15 +851,15 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Café da manhã com Gracinha</t>
+          <t>Alimentos e Materiais de limpeza</t>
         </is>
       </c>
       <c r="C10" s="3" t="n">
-        <v>-98.5</v>
+        <v>-97.89</v>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Restaurante</t>
+          <t>Supermercado</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
@@ -894,20 +894,20 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Alimentos e Materiais de limpeza</t>
+          <t>Ajuda a Casa do Pobre</t>
         </is>
       </c>
       <c r="C11" s="3" t="n">
-        <v>-97.89</v>
+        <v>-30</v>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Supermercado</t>
+          <t>Doações e Ajudas</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Cartão BB VISA</t>
+          <t>Conta BB</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
@@ -917,12 +917,12 @@
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>ALIMENTAÇÃO E LIMPEZA</t>
+          <t>DOAÇÕES</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>Despesas com alimentação e limpeza</t>
+          <t>Despesas com doações</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
@@ -937,15 +937,15 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Ajuda a Casa do Pobre</t>
+          <t>Hotel Real Classic para IPD</t>
         </is>
       </c>
       <c r="C12" s="3" t="n">
-        <v>-30</v>
+        <v>-94.56</v>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Doações e Ajudas</t>
+          <t>VIAGENS/Estadia</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
@@ -960,12 +960,17 @@
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>DOAÇÕES</t>
+          <t>LAZER</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>VIAGENS</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>Despesas com doações</t>
+          <t>Despesas com lazer</t>
         </is>
       </c>
       <c r="J12" t="inlineStr">
@@ -980,15 +985,15 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Ovos</t>
+          <t>Café da manhã com Gracinha</t>
         </is>
       </c>
       <c r="C13" s="3" t="n">
-        <v>-15.5</v>
+        <v>-98.5</v>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Padaria</t>
+          <t>Restaurante</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
@@ -1023,20 +1028,20 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Hotel Real Classic para IPD</t>
+          <t>Ovos</t>
         </is>
       </c>
       <c r="C14" s="3" t="n">
-        <v>-94.56</v>
+        <v>-15.5</v>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>VIAGENS/Estadia</t>
+          <t>Padaria</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Conta BB</t>
+          <t>Cartão BB VISA</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
@@ -1046,17 +1051,12 @@
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>LAZER</t>
-        </is>
-      </c>
-      <c r="H14" t="inlineStr">
-        <is>
-          <t>VIAGENS</t>
+          <t>ALIMENTAÇÃO E LIMPEZA</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>Despesas com lazer</t>
+          <t>Despesas com alimentação e limpeza</t>
         </is>
       </c>
       <c r="J14" t="inlineStr">
@@ -36283,11 +36283,11 @@
       </c>
       <c r="B809" t="inlineStr">
         <is>
-          <t>Casa Aracaju -  Peças para o conserto bomba do jardim</t>
+          <t>Casa Aracaju - Conserto da Bomba do jardim</t>
         </is>
       </c>
       <c r="C809" s="3" t="n">
-        <v>-26.5</v>
+        <v>-250</v>
       </c>
       <c r="D809" t="inlineStr">
         <is>
@@ -36296,7 +36296,7 @@
       </c>
       <c r="E809" t="inlineStr">
         <is>
-          <t>Cartão BB VISA</t>
+          <t>Conta BB</t>
         </is>
       </c>
       <c r="F809" t="inlineStr">
@@ -36675,11 +36675,11 @@
       </c>
       <c r="B818" t="inlineStr">
         <is>
-          <t>Casa Aracaju - Conserto da Bomba do jardim</t>
+          <t>Casa Aracaju -  Peças para o conserto bomba do jardim</t>
         </is>
       </c>
       <c r="C818" s="3" t="n">
-        <v>-250</v>
+        <v>-26.5</v>
       </c>
       <c r="D818" t="inlineStr">
         <is>
@@ -36688,7 +36688,7 @@
       </c>
       <c r="E818" t="inlineStr">
         <is>
-          <t>Conta BB</t>
+          <t>Cartão BB VISA</t>
         </is>
       </c>
       <c r="F818" t="inlineStr">
@@ -36938,20 +36938,20 @@
       </c>
       <c r="B824" t="inlineStr">
         <is>
-          <t>Ajuda a Casa do Pobre</t>
+          <t>Café da manhã</t>
         </is>
       </c>
       <c r="C824" s="3" t="n">
-        <v>-30</v>
+        <v>-38.83</v>
       </c>
       <c r="D824" t="inlineStr">
         <is>
-          <t>Doações e Ajudas</t>
+          <t>Restaurante</t>
         </is>
       </c>
       <c r="E824" t="inlineStr">
         <is>
-          <t>Conta BB</t>
+          <t>Cartão BB VISA</t>
         </is>
       </c>
       <c r="F824" t="inlineStr">
@@ -36961,12 +36961,12 @@
       </c>
       <c r="G824" t="inlineStr">
         <is>
-          <t>DOAÇÕES</t>
+          <t>ALIMENTAÇÃO E LIMPEZA</t>
         </is>
       </c>
       <c r="I824" t="inlineStr">
         <is>
-          <t>Despesas com doações</t>
+          <t>Despesas com alimentação e limpeza</t>
         </is>
       </c>
       <c r="J824" t="inlineStr">
@@ -37029,20 +37029,20 @@
       </c>
       <c r="B826" t="inlineStr">
         <is>
-          <t>Café da manhã</t>
+          <t>Ajuda a Casa do Pobre</t>
         </is>
       </c>
       <c r="C826" s="3" t="n">
-        <v>-38.83</v>
+        <v>-30</v>
       </c>
       <c r="D826" t="inlineStr">
         <is>
-          <t>Restaurante</t>
+          <t>Doações e Ajudas</t>
         </is>
       </c>
       <c r="E826" t="inlineStr">
         <is>
-          <t>Cartão BB VISA</t>
+          <t>Conta BB</t>
         </is>
       </c>
       <c r="F826" t="inlineStr">
@@ -37052,12 +37052,12 @@
       </c>
       <c r="G826" t="inlineStr">
         <is>
-          <t>ALIMENTAÇÃO E LIMPEZA</t>
+          <t>DOAÇÕES</t>
         </is>
       </c>
       <c r="I826" t="inlineStr">
         <is>
-          <t>Despesas com alimentação e limpeza</t>
+          <t>Despesas com doações</t>
         </is>
       </c>
       <c r="J826" t="inlineStr">
@@ -54809,20 +54809,20 @@
       </c>
       <c r="B1226" t="inlineStr">
         <is>
-          <t>Alimentos e Materiais de limpeza (10 / 10)</t>
+          <t>Perfume no Boticário (2 / 10)</t>
         </is>
       </c>
       <c r="C1226" s="3" t="n">
-        <v>-24.8</v>
+        <v>-8.99</v>
       </c>
       <c r="D1226" t="inlineStr">
         <is>
-          <t>Supermercado</t>
+          <t>Salão de Beleza e Cosméticos</t>
         </is>
       </c>
       <c r="E1226" t="inlineStr">
         <is>
-          <t>Cartão BB ELO</t>
+          <t>Cartão BB VISA</t>
         </is>
       </c>
       <c r="F1226" t="inlineStr">
@@ -54832,12 +54832,12 @@
       </c>
       <c r="G1226" t="inlineStr">
         <is>
-          <t>ALIMENTAÇÃO E LIMPEZA</t>
+          <t>FAMÍLIA</t>
         </is>
       </c>
       <c r="I1226" t="inlineStr">
         <is>
-          <t>Despesas com alimentação e limpeza</t>
+          <t>Despesas com família</t>
         </is>
       </c>
       <c r="J1226" t="inlineStr">
@@ -54852,20 +54852,20 @@
       </c>
       <c r="B1227" t="inlineStr">
         <is>
-          <t>Perfume no Boticário (2 / 10)</t>
+          <t>Alimentos e Materiais de limpeza (10 / 10)</t>
         </is>
       </c>
       <c r="C1227" s="3" t="n">
-        <v>-8.99</v>
+        <v>-24.8</v>
       </c>
       <c r="D1227" t="inlineStr">
         <is>
-          <t>Salão de Beleza e Cosméticos</t>
+          <t>Supermercado</t>
         </is>
       </c>
       <c r="E1227" t="inlineStr">
         <is>
-          <t>Cartão BB VISA</t>
+          <t>Cartão BB ELO</t>
         </is>
       </c>
       <c r="F1227" t="inlineStr">
@@ -54875,12 +54875,12 @@
       </c>
       <c r="G1227" t="inlineStr">
         <is>
-          <t>FAMÍLIA</t>
+          <t>ALIMENTAÇÃO E LIMPEZA</t>
         </is>
       </c>
       <c r="I1227" t="inlineStr">
         <is>
-          <t>Despesas com família</t>
+          <t>Despesas com alimentação e limpeza</t>
         </is>
       </c>
       <c r="J1227" t="inlineStr">
@@ -63861,20 +63861,20 @@
       </c>
       <c r="B1430" t="inlineStr">
         <is>
-          <t>Casa Aracaju - Energia Elétrica</t>
+          <t>Rendimentos Saldo Conta WISE</t>
         </is>
       </c>
       <c r="C1430" s="3" t="n">
-        <v>-213.57</v>
+        <v>37.28</v>
       </c>
       <c r="D1430" t="inlineStr">
         <is>
-          <t>Energia Elétrica</t>
+          <t>Juros de Investimento</t>
         </is>
       </c>
       <c r="E1430" t="inlineStr">
         <is>
-          <t>Conta BB</t>
+          <t>Cartão WISE</t>
         </is>
       </c>
       <c r="F1430" t="inlineStr">
@@ -63884,22 +63884,22 @@
       </c>
       <c r="G1430" t="inlineStr">
         <is>
-          <t>IMÓVEIS</t>
+          <t>RECEITAS</t>
         </is>
       </c>
       <c r="H1430" t="inlineStr">
         <is>
-          <t>Contas da casa</t>
+          <t>Financeiras</t>
         </is>
       </c>
       <c r="I1430" t="inlineStr">
         <is>
-          <t>Despesas com imóveis</t>
+          <t>Receitas Financeiras</t>
         </is>
       </c>
       <c r="J1430" t="inlineStr">
         <is>
-          <t>Despesas e Custos</t>
+          <t>Receitas Financeiras</t>
         </is>
       </c>
     </row>
@@ -64086,20 +64086,20 @@
       </c>
       <c r="B1435" t="inlineStr">
         <is>
-          <t>Rendimentos Saldo Conta WISE</t>
+          <t>Casa Aracaju - Energia Elétrica</t>
         </is>
       </c>
       <c r="C1435" s="3" t="n">
-        <v>37.28</v>
+        <v>-213.57</v>
       </c>
       <c r="D1435" t="inlineStr">
         <is>
-          <t>Juros de Investimento</t>
+          <t>Energia Elétrica</t>
         </is>
       </c>
       <c r="E1435" t="inlineStr">
         <is>
-          <t>Cartão WISE</t>
+          <t>Conta BB</t>
         </is>
       </c>
       <c r="F1435" t="inlineStr">
@@ -64109,22 +64109,22 @@
       </c>
       <c r="G1435" t="inlineStr">
         <is>
-          <t>RECEITAS</t>
+          <t>IMÓVEIS</t>
         </is>
       </c>
       <c r="H1435" t="inlineStr">
         <is>
-          <t>Financeiras</t>
+          <t>Contas da casa</t>
         </is>
       </c>
       <c r="I1435" t="inlineStr">
         <is>
-          <t>Receitas Financeiras</t>
+          <t>Despesas com imóveis</t>
         </is>
       </c>
       <c r="J1435" t="inlineStr">
         <is>
-          <t>Receitas Financeiras</t>
+          <t>Despesas e Custos</t>
         </is>
       </c>
     </row>
@@ -64230,15 +64230,15 @@
       </c>
       <c r="B1438" t="inlineStr">
         <is>
-          <t>Garafas de água</t>
+          <t>Remédios para ACMD</t>
         </is>
       </c>
       <c r="C1438" s="3" t="n">
-        <v>-14</v>
+        <v>-93.98999999999999</v>
       </c>
       <c r="D1438" t="inlineStr">
         <is>
-          <t>VIAGENS/Alimentação</t>
+          <t>Farmácia</t>
         </is>
       </c>
       <c r="E1438" t="inlineStr">
@@ -64253,17 +64253,12 @@
       </c>
       <c r="G1438" t="inlineStr">
         <is>
-          <t>LAZER</t>
-        </is>
-      </c>
-      <c r="H1438" t="inlineStr">
-        <is>
-          <t>VIAGENS</t>
+          <t>SAÚDE</t>
         </is>
       </c>
       <c r="I1438" t="inlineStr">
         <is>
-          <t>Despesas com lazer</t>
+          <t>Despesas com Saúde</t>
         </is>
       </c>
       <c r="J1438" t="inlineStr">
@@ -64278,15 +64273,15 @@
       </c>
       <c r="B1439" t="inlineStr">
         <is>
-          <t>Remédios para ACMD</t>
+          <t>Garafas de água</t>
         </is>
       </c>
       <c r="C1439" s="3" t="n">
-        <v>-93.98999999999999</v>
+        <v>-14</v>
       </c>
       <c r="D1439" t="inlineStr">
         <is>
-          <t>Farmácia</t>
+          <t>VIAGENS/Alimentação</t>
         </is>
       </c>
       <c r="E1439" t="inlineStr">
@@ -64301,12 +64296,17 @@
       </c>
       <c r="G1439" t="inlineStr">
         <is>
-          <t>SAÚDE</t>
+          <t>LAZER</t>
+        </is>
+      </c>
+      <c r="H1439" t="inlineStr">
+        <is>
+          <t>VIAGENS</t>
         </is>
       </c>
       <c r="I1439" t="inlineStr">
         <is>
-          <t>Despesas com Saúde</t>
+          <t>Despesas com lazer</t>
         </is>
       </c>
       <c r="J1439" t="inlineStr">
@@ -68928,11 +68928,11 @@
       </c>
       <c r="B1544" t="inlineStr">
         <is>
-          <t>Benefício PETROS II</t>
+          <t>Benefício PETROS</t>
         </is>
       </c>
       <c r="C1544" s="3" t="n">
-        <v>4694.46</v>
+        <v>10524.94</v>
       </c>
       <c r="D1544" t="inlineStr">
         <is>
@@ -69024,11 +69024,11 @@
       </c>
       <c r="B1546" t="inlineStr">
         <is>
-          <t>Benefício PETROS</t>
+          <t>Benefício PETROS II</t>
         </is>
       </c>
       <c r="C1546" s="3" t="n">
-        <v>10524.94</v>
+        <v>4694.46</v>
       </c>
       <c r="D1546" t="inlineStr">
         <is>
@@ -69163,15 +69163,15 @@
       </c>
       <c r="B1549" t="inlineStr">
         <is>
-          <t>Passagem GRU / AJU - ACMD e MGAP - 21/11/2026 (2 / 2)</t>
+          <t>Link de Internet - CLARO</t>
         </is>
       </c>
       <c r="C1549" s="3" t="n">
-        <v>-312</v>
+        <v>-267.06</v>
       </c>
       <c r="D1549" t="inlineStr">
         <is>
-          <t>VIAGENS/Passagens</t>
+          <t>Internet</t>
         </is>
       </c>
       <c r="E1549" t="inlineStr">
@@ -69186,17 +69186,12 @@
       </c>
       <c r="G1549" t="inlineStr">
         <is>
-          <t>LAZER</t>
-        </is>
-      </c>
-      <c r="H1549" t="inlineStr">
-        <is>
-          <t>VIAGENS</t>
+          <t>TECNOLOGIA E COMUNICAÇÃO</t>
         </is>
       </c>
       <c r="I1549" t="inlineStr">
         <is>
-          <t>Despesas com lazer</t>
+          <t>Despesas com TI</t>
         </is>
       </c>
       <c r="J1549" t="inlineStr">
@@ -69211,20 +69206,20 @@
       </c>
       <c r="B1550" t="inlineStr">
         <is>
-          <t>Salada de frutas</t>
+          <t>Pagamento "DUO GOURMET"</t>
         </is>
       </c>
       <c r="C1550" s="3" t="n">
-        <v>-29.15</v>
+        <v>-45</v>
       </c>
       <c r="D1550" t="inlineStr">
         <is>
-          <t>Lanchonete</t>
+          <t>Restaurante</t>
         </is>
       </c>
       <c r="E1550" t="inlineStr">
         <is>
-          <t>Cartão BB VISA</t>
+          <t>Conta BB</t>
         </is>
       </c>
       <c r="F1550" t="inlineStr">
@@ -69254,15 +69249,15 @@
       </c>
       <c r="B1551" t="inlineStr">
         <is>
-          <t>Link de Internet - CLARO</t>
+          <t>Passagem GRU / AJU - ACMD e MGAP - 21/11/2026 (2 / 2)</t>
         </is>
       </c>
       <c r="C1551" s="3" t="n">
-        <v>-267.06</v>
+        <v>-312</v>
       </c>
       <c r="D1551" t="inlineStr">
         <is>
-          <t>Internet</t>
+          <t>VIAGENS/Passagens</t>
         </is>
       </c>
       <c r="E1551" t="inlineStr">
@@ -69277,12 +69272,17 @@
       </c>
       <c r="G1551" t="inlineStr">
         <is>
-          <t>TECNOLOGIA E COMUNICAÇÃO</t>
+          <t>LAZER</t>
+        </is>
+      </c>
+      <c r="H1551" t="inlineStr">
+        <is>
+          <t>VIAGENS</t>
         </is>
       </c>
       <c r="I1551" t="inlineStr">
         <is>
-          <t>Despesas com TI</t>
+          <t>Despesas com lazer</t>
         </is>
       </c>
       <c r="J1551" t="inlineStr">
@@ -69297,20 +69297,20 @@
       </c>
       <c r="B1552" t="inlineStr">
         <is>
-          <t>Pagamento "DUO GOURMET"</t>
+          <t>Salada de frutas</t>
         </is>
       </c>
       <c r="C1552" s="3" t="n">
-        <v>-45</v>
+        <v>-29.15</v>
       </c>
       <c r="D1552" t="inlineStr">
         <is>
-          <t>Restaurante</t>
+          <t>Lanchonete</t>
         </is>
       </c>
       <c r="E1552" t="inlineStr">
         <is>
-          <t>Conta BB</t>
+          <t>Cartão BB VISA</t>
         </is>
       </c>
       <c r="F1552" t="inlineStr">
@@ -69340,20 +69340,20 @@
       </c>
       <c r="B1553" t="inlineStr">
         <is>
-          <t>Combustível para RANGER XLT</t>
+          <t>Apt.AJU. - Investimento Cozinha</t>
         </is>
       </c>
       <c r="C1553" s="3" t="n">
-        <v>-364.5</v>
+        <v>-1500</v>
       </c>
       <c r="D1553" t="inlineStr">
         <is>
-          <t>Combustível</t>
+          <t>Ampliação-Melhorias Imóveis</t>
         </is>
       </c>
       <c r="E1553" t="inlineStr">
         <is>
-          <t>Cartão BB VISA</t>
+          <t>Conta BB</t>
         </is>
       </c>
       <c r="F1553" t="inlineStr">
@@ -69363,17 +69363,17 @@
       </c>
       <c r="G1553" t="inlineStr">
         <is>
-          <t>TRANSPORTE</t>
+          <t>BENS DURÁVEIS</t>
         </is>
       </c>
       <c r="I1553" t="inlineStr">
         <is>
-          <t>Despesas com Combustível</t>
+          <t>Investimentos Bens Imóveis</t>
         </is>
       </c>
       <c r="J1553" t="inlineStr">
         <is>
-          <t>Despesas e Custos</t>
+          <t>Investimentos Bens Imóveis</t>
         </is>
       </c>
     </row>
@@ -69383,15 +69383,15 @@
       </c>
       <c r="B1554" t="inlineStr">
         <is>
-          <t>Troca da bateria do MACBOOK PRO</t>
+          <t>Combustível para RANGER XLT</t>
         </is>
       </c>
       <c r="C1554" s="3" t="n">
-        <v>-102.5</v>
+        <v>-364.5</v>
       </c>
       <c r="D1554" t="inlineStr">
         <is>
-          <t>OUTRAS DESPESAS</t>
+          <t>Combustível</t>
         </is>
       </c>
       <c r="E1554" t="inlineStr">
@@ -69406,12 +69406,12 @@
       </c>
       <c r="G1554" t="inlineStr">
         <is>
-          <t>OUTRAS DESPESAS</t>
+          <t>TRANSPORTE</t>
         </is>
       </c>
       <c r="I1554" t="inlineStr">
         <is>
-          <t>Outras Despesas</t>
+          <t>Despesas com Combustível</t>
         </is>
       </c>
       <c r="J1554" t="inlineStr">
@@ -69426,15 +69426,15 @@
       </c>
       <c r="B1555" t="inlineStr">
         <is>
-          <t>Aquisição do celular MOTOROLA G86</t>
+          <t>Troca da bateria do MACBOOK PRO</t>
         </is>
       </c>
       <c r="C1555" s="3" t="n">
-        <v>-139</v>
+        <v>-102.5</v>
       </c>
       <c r="D1555" t="inlineStr">
         <is>
-          <t>Eletrônicos</t>
+          <t>OUTRAS DESPESAS</t>
         </is>
       </c>
       <c r="E1555" t="inlineStr">
@@ -69449,17 +69449,17 @@
       </c>
       <c r="G1555" t="inlineStr">
         <is>
-          <t>BENS DURÁVEIS</t>
+          <t>OUTRAS DESPESAS</t>
         </is>
       </c>
       <c r="I1555" t="inlineStr">
         <is>
-          <t>Investimentos Bens</t>
+          <t>Outras Despesas</t>
         </is>
       </c>
       <c r="J1555" t="inlineStr">
         <is>
-          <t>Investimentos</t>
+          <t>Despesas e Custos</t>
         </is>
       </c>
     </row>
@@ -69469,20 +69469,20 @@
       </c>
       <c r="B1556" t="inlineStr">
         <is>
-          <t>Apt.AJU. - Investimento Cozinha</t>
+          <t>Aquisição do celular MOTOROLA G86</t>
         </is>
       </c>
       <c r="C1556" s="3" t="n">
-        <v>-1500</v>
+        <v>-139</v>
       </c>
       <c r="D1556" t="inlineStr">
         <is>
-          <t>Ampliação-Melhorias Imóveis</t>
+          <t>Eletrônicos</t>
         </is>
       </c>
       <c r="E1556" t="inlineStr">
         <is>
-          <t>Conta BB</t>
+          <t>Cartão BB VISA</t>
         </is>
       </c>
       <c r="F1556" t="inlineStr">
@@ -69497,12 +69497,12 @@
       </c>
       <c r="I1556" t="inlineStr">
         <is>
-          <t>Investimentos Bens Imóveis</t>
+          <t>Investimentos Bens</t>
         </is>
       </c>
       <c r="J1556" t="inlineStr">
         <is>
-          <t>Investimentos Bens Imóveis</t>
+          <t>Investimentos</t>
         </is>
       </c>
     </row>
@@ -69512,20 +69512,20 @@
       </c>
       <c r="B1557" t="inlineStr">
         <is>
-          <t>TV SAMSUNG quarto do casal (6 / 8)</t>
+          <t>Apt. SP. - Gás Natural</t>
         </is>
       </c>
       <c r="C1557" s="3" t="n">
-        <v>-337.49</v>
+        <v>-63.96</v>
       </c>
       <c r="D1557" t="inlineStr">
         <is>
-          <t>Acessórios</t>
+          <t>Gás</t>
         </is>
       </c>
       <c r="E1557" t="inlineStr">
         <is>
-          <t>Cartão BB VISA</t>
+          <t>Conta BB</t>
         </is>
       </c>
       <c r="F1557" t="inlineStr">
@@ -69535,12 +69535,17 @@
       </c>
       <c r="G1557" t="inlineStr">
         <is>
-          <t>FAMÍLIA</t>
+          <t>IMÓVEIS</t>
+        </is>
+      </c>
+      <c r="H1557" t="inlineStr">
+        <is>
+          <t>Contas da casa</t>
         </is>
       </c>
       <c r="I1557" t="inlineStr">
         <is>
-          <t>Despesas com família</t>
+          <t>Despesas com imóveis</t>
         </is>
       </c>
       <c r="J1557" t="inlineStr">
@@ -69598,35 +69603,35 @@
       </c>
       <c r="B1559" t="inlineStr">
         <is>
-          <t>Estacionamento</t>
+          <t>TV SAMSUNG quarto do casal (6 / 8)</t>
         </is>
       </c>
       <c r="C1559" s="3" t="n">
-        <v>-5</v>
+        <v>-337.49</v>
       </c>
       <c r="D1559" t="inlineStr">
         <is>
-          <t>Estacionamento</t>
+          <t>Acessórios</t>
         </is>
       </c>
       <c r="E1559" t="inlineStr">
         <is>
-          <t>Conta BB</t>
+          <t>Cartão BB VISA</t>
         </is>
       </c>
       <c r="F1559" t="inlineStr">
         <is>
-          <t>Sim</t>
+          <t>Não</t>
         </is>
       </c>
       <c r="G1559" t="inlineStr">
         <is>
-          <t>TRANSPORTE</t>
+          <t>FAMÍLIA</t>
         </is>
       </c>
       <c r="I1559" t="inlineStr">
         <is>
-          <t>Despesas com Estacionamento</t>
+          <t>Despesas com família</t>
         </is>
       </c>
       <c r="J1559" t="inlineStr">
@@ -69641,15 +69646,15 @@
       </c>
       <c r="B1560" t="inlineStr">
         <is>
-          <t>Apt. SP. - Gás Natural</t>
+          <t>Estacionamento</t>
         </is>
       </c>
       <c r="C1560" s="3" t="n">
-        <v>-63.96</v>
+        <v>-5</v>
       </c>
       <c r="D1560" t="inlineStr">
         <is>
-          <t>Gás</t>
+          <t>Estacionamento</t>
         </is>
       </c>
       <c r="E1560" t="inlineStr">
@@ -69659,22 +69664,17 @@
       </c>
       <c r="F1560" t="inlineStr">
         <is>
-          <t>Não</t>
+          <t>Sim</t>
         </is>
       </c>
       <c r="G1560" t="inlineStr">
         <is>
-          <t>IMÓVEIS</t>
-        </is>
-      </c>
-      <c r="H1560" t="inlineStr">
-        <is>
-          <t>Contas da casa</t>
+          <t>TRANSPORTE</t>
         </is>
       </c>
       <c r="I1560" t="inlineStr">
         <is>
-          <t>Despesas com imóveis</t>
+          <t>Despesas com Estacionamento</t>
         </is>
       </c>
       <c r="J1560" t="inlineStr">
@@ -69728,24 +69728,24 @@
     </row>
     <row r="1562">
       <c r="A1562" s="2" t="n">
-        <v>46325</v>
+        <v>46324</v>
       </c>
       <c r="B1562" t="inlineStr">
         <is>
-          <t>Casa Aracaju - Água e Esgoto</t>
+          <t>Alimentos</t>
         </is>
       </c>
       <c r="C1562" s="3" t="n">
-        <v>-108.5</v>
+        <v>-205.07</v>
       </c>
       <c r="D1562" t="inlineStr">
         <is>
-          <t>Água e Esgoto</t>
+          <t>Supermercado</t>
         </is>
       </c>
       <c r="E1562" t="inlineStr">
         <is>
-          <t>Conta BB</t>
+          <t>Cartão BB VISA</t>
         </is>
       </c>
       <c r="F1562" t="inlineStr">
@@ -69755,17 +69755,12 @@
       </c>
       <c r="G1562" t="inlineStr">
         <is>
-          <t>IMÓVEIS</t>
-        </is>
-      </c>
-      <c r="H1562" t="inlineStr">
-        <is>
-          <t>Contas da casa</t>
+          <t>ALIMENTAÇÃO E LIMPEZA</t>
         </is>
       </c>
       <c r="I1562" t="inlineStr">
         <is>
-          <t>Despesas com imóveis</t>
+          <t>Despesas com alimentação e limpeza</t>
         </is>
       </c>
       <c r="J1562" t="inlineStr">
@@ -69776,24 +69771,24 @@
     </row>
     <row r="1563">
       <c r="A1563" s="2" t="n">
-        <v>46327</v>
+        <v>46324</v>
       </c>
       <c r="B1563" t="inlineStr">
         <is>
-          <t>Seguro Apt Aracaju - Parcelas 3</t>
+          <t>Almoço com Gracinha</t>
         </is>
       </c>
       <c r="C1563" s="3" t="n">
-        <v>-52.85</v>
+        <v>-228.5</v>
       </c>
       <c r="D1563" t="inlineStr">
         <is>
-          <t>Residencial</t>
+          <t>Restaurante</t>
         </is>
       </c>
       <c r="E1563" t="inlineStr">
         <is>
-          <t>Conta BB</t>
+          <t>Cartão BB VISA</t>
         </is>
       </c>
       <c r="F1563" t="inlineStr">
@@ -69803,12 +69798,12 @@
       </c>
       <c r="G1563" t="inlineStr">
         <is>
-          <t>SEGUROS E SERVIÇOS FUNERÁRIOS</t>
+          <t>ALIMENTAÇÃO E LIMPEZA</t>
         </is>
       </c>
       <c r="I1563" t="inlineStr">
         <is>
-          <t>Despesas com Seguros</t>
+          <t>Despesas com alimentação e limpeza</t>
         </is>
       </c>
       <c r="J1563" t="inlineStr">
@@ -69819,19 +69814,19 @@
     </row>
     <row r="1564">
       <c r="A1564" s="2" t="n">
-        <v>46327</v>
+        <v>46325</v>
       </c>
       <c r="B1564" t="inlineStr">
         <is>
-          <t>Cemitério Colina da Saudade 2026</t>
+          <t>Casa Aracaju - Água e Esgoto</t>
         </is>
       </c>
       <c r="C1564" s="3" t="n">
-        <v>-600</v>
+        <v>-108.5</v>
       </c>
       <c r="D1564" t="inlineStr">
         <is>
-          <t>Serviços Funerários</t>
+          <t>Água e Esgoto</t>
         </is>
       </c>
       <c r="E1564" t="inlineStr">
@@ -69846,12 +69841,17 @@
       </c>
       <c r="G1564" t="inlineStr">
         <is>
-          <t>SEGUROS E SERVIÇOS FUNERÁRIOS</t>
+          <t>IMÓVEIS</t>
+        </is>
+      </c>
+      <c r="H1564" t="inlineStr">
+        <is>
+          <t>Contas da casa</t>
         </is>
       </c>
       <c r="I1564" t="inlineStr">
         <is>
-          <t>Despesas com Seguros</t>
+          <t>Despesas com imóveis</t>
         </is>
       </c>
       <c r="J1564" t="inlineStr">
@@ -69862,19 +69862,19 @@
     </row>
     <row r="1565">
       <c r="A1565" s="2" t="n">
-        <v>46328</v>
+        <v>46327</v>
       </c>
       <c r="B1565" t="inlineStr">
         <is>
-          <t>Seguro de Itens Pessoais</t>
+          <t>Cemitério Colina da Saudade 2026</t>
         </is>
       </c>
       <c r="C1565" s="3" t="n">
-        <v>-9.9</v>
+        <v>-600</v>
       </c>
       <c r="D1565" t="inlineStr">
         <is>
-          <t>Equipamentos Eletrônicos</t>
+          <t>Serviços Funerários</t>
         </is>
       </c>
       <c r="E1565" t="inlineStr">
@@ -69905,19 +69905,19 @@
     </row>
     <row r="1566">
       <c r="A1566" s="2" t="n">
-        <v>46329</v>
+        <v>46327</v>
       </c>
       <c r="B1566" t="inlineStr">
         <is>
-          <t>Casa Aracaju - Energia Elétrica</t>
+          <t>Seguro Apt Aracaju - Parcelas 3</t>
         </is>
       </c>
       <c r="C1566" s="3" t="n">
-        <v>-182</v>
+        <v>-52.85</v>
       </c>
       <c r="D1566" t="inlineStr">
         <is>
-          <t>Energia Elétrica</t>
+          <t>Residencial</t>
         </is>
       </c>
       <c r="E1566" t="inlineStr">
@@ -69932,17 +69932,12 @@
       </c>
       <c r="G1566" t="inlineStr">
         <is>
-          <t>IMÓVEIS</t>
-        </is>
-      </c>
-      <c r="H1566" t="inlineStr">
-        <is>
-          <t>Contas da casa</t>
+          <t>SEGUROS E SERVIÇOS FUNERÁRIOS</t>
         </is>
       </c>
       <c r="I1566" t="inlineStr">
         <is>
-          <t>Despesas com imóveis</t>
+          <t>Despesas com Seguros</t>
         </is>
       </c>
       <c r="J1566" t="inlineStr">
@@ -69953,19 +69948,19 @@
     </row>
     <row r="1567">
       <c r="A1567" s="2" t="n">
-        <v>46329</v>
+        <v>46328</v>
       </c>
       <c r="B1567" t="inlineStr">
         <is>
-          <t>Apt. Aju. - Energia Elétrica</t>
+          <t>Seguro de Itens Pessoais</t>
         </is>
       </c>
       <c r="C1567" s="3" t="n">
-        <v>-169.78</v>
+        <v>-9.9</v>
       </c>
       <c r="D1567" t="inlineStr">
         <is>
-          <t>Energia Elétrica</t>
+          <t>Equipamentos Eletrônicos</t>
         </is>
       </c>
       <c r="E1567" t="inlineStr">
@@ -69980,17 +69975,12 @@
       </c>
       <c r="G1567" t="inlineStr">
         <is>
-          <t>IMÓVEIS</t>
-        </is>
-      </c>
-      <c r="H1567" t="inlineStr">
-        <is>
-          <t>Contas da casa</t>
+          <t>SEGUROS E SERVIÇOS FUNERÁRIOS</t>
         </is>
       </c>
       <c r="I1567" t="inlineStr">
         <is>
-          <t>Despesas com imóveis</t>
+          <t>Despesas com Seguros</t>
         </is>
       </c>
       <c r="J1567" t="inlineStr">
@@ -70005,15 +69995,15 @@
       </c>
       <c r="B1568" t="inlineStr">
         <is>
-          <t>Resgate Parcial BB Deb Inc CDI Pvt</t>
+          <t>Casa Aracaju - Energia Elétrica</t>
         </is>
       </c>
       <c r="C1568" s="3" t="n">
-        <v>200000</v>
+        <v>-182</v>
       </c>
       <c r="D1568" t="inlineStr">
         <is>
-          <t>Resgate de Investimento</t>
+          <t>Energia Elétrica</t>
         </is>
       </c>
       <c r="E1568" t="inlineStr">
@@ -70028,35 +70018,40 @@
       </c>
       <c r="G1568" t="inlineStr">
         <is>
-          <t>INVESTIMENTOS E PATRIMÔNIO</t>
+          <t>IMÓVEIS</t>
+        </is>
+      </c>
+      <c r="H1568" t="inlineStr">
+        <is>
+          <t>Contas da casa</t>
         </is>
       </c>
       <c r="I1568" t="inlineStr">
         <is>
-          <t>Receitas Financeiras</t>
+          <t>Despesas com imóveis</t>
         </is>
       </c>
       <c r="J1568" t="inlineStr">
         <is>
-          <t>Receitas Financeiras</t>
+          <t>Despesas e Custos</t>
         </is>
       </c>
     </row>
     <row r="1569">
       <c r="A1569" s="2" t="n">
-        <v>46332</v>
+        <v>46329</v>
       </c>
       <c r="B1569" t="inlineStr">
         <is>
-          <t>Casa Aracaju - Aquisição e instalação da piscina</t>
+          <t>Apt. Aju. - Energia Elétrica</t>
         </is>
       </c>
       <c r="C1569" s="3" t="n">
-        <v>-17600</v>
+        <v>-169.78</v>
       </c>
       <c r="D1569" t="inlineStr">
         <is>
-          <t>Ampliação-Melhorias Imóveis</t>
+          <t>Energia Elétrica</t>
         </is>
       </c>
       <c r="E1569" t="inlineStr">
@@ -70071,40 +70066,45 @@
       </c>
       <c r="G1569" t="inlineStr">
         <is>
-          <t>BENS DURÁVEIS</t>
+          <t>IMÓVEIS</t>
+        </is>
+      </c>
+      <c r="H1569" t="inlineStr">
+        <is>
+          <t>Contas da casa</t>
         </is>
       </c>
       <c r="I1569" t="inlineStr">
         <is>
-          <t>Investimentos Bens Imóveis</t>
+          <t>Despesas com imóveis</t>
         </is>
       </c>
       <c r="J1569" t="inlineStr">
         <is>
-          <t>Investimentos Bens Imóveis</t>
+          <t>Despesas e Custos</t>
         </is>
       </c>
     </row>
     <row r="1570">
       <c r="A1570" s="2" t="n">
-        <v>46332</v>
+        <v>46329</v>
       </c>
       <c r="B1570" t="inlineStr">
         <is>
-          <t>Película para RANGER XLT</t>
+          <t>Resgate Parcial BB Deb Inc CDI Pvt</t>
         </is>
       </c>
       <c r="C1570" s="3" t="n">
-        <v>-100</v>
+        <v>200000</v>
       </c>
       <c r="D1570" t="inlineStr">
         <is>
-          <t>Automóvel/Manutenção</t>
+          <t>Resgate de Investimento</t>
         </is>
       </c>
       <c r="E1570" t="inlineStr">
         <is>
-          <t>Cartão BB VISA</t>
+          <t>Conta BB</t>
         </is>
       </c>
       <c r="F1570" t="inlineStr">
@@ -70114,22 +70114,17 @@
       </c>
       <c r="G1570" t="inlineStr">
         <is>
-          <t>TRANSPORTE</t>
-        </is>
-      </c>
-      <c r="H1570" t="inlineStr">
-        <is>
-          <t>Automóvel</t>
+          <t>INVESTIMENTOS E PATRIMÔNIO</t>
         </is>
       </c>
       <c r="I1570" t="inlineStr">
         <is>
-          <t>Despesas com Automóvel (Manutenção)</t>
+          <t>Receitas Financeiras</t>
         </is>
       </c>
       <c r="J1570" t="inlineStr">
         <is>
-          <t>Despesas e Custos</t>
+          <t>Receitas Financeiras</t>
         </is>
       </c>
     </row>
@@ -70139,20 +70134,20 @@
       </c>
       <c r="B1571" t="inlineStr">
         <is>
-          <t>Filtro para a COIFA - CONSUL</t>
+          <t>Casa Aracaju - Aquisição e instalação da piscina</t>
         </is>
       </c>
       <c r="C1571" s="3" t="n">
-        <v>-138.27</v>
+        <v>-17600</v>
       </c>
       <c r="D1571" t="inlineStr">
         <is>
-          <t>Restauração e Manutenção</t>
+          <t>Ampliação-Melhorias Imóveis</t>
         </is>
       </c>
       <c r="E1571" t="inlineStr">
         <is>
-          <t>Cartão BB ELO</t>
+          <t>Conta BB</t>
         </is>
       </c>
       <c r="F1571" t="inlineStr">
@@ -70162,45 +70157,40 @@
       </c>
       <c r="G1571" t="inlineStr">
         <is>
-          <t>IMÓVEIS</t>
-        </is>
-      </c>
-      <c r="H1571" t="inlineStr">
-        <is>
-          <t>Manutenção e encargos</t>
+          <t>BENS DURÁVEIS</t>
         </is>
       </c>
       <c r="I1571" t="inlineStr">
         <is>
-          <t>Despesas com imóveis</t>
+          <t>Investimentos Bens Imóveis</t>
         </is>
       </c>
       <c r="J1571" t="inlineStr">
         <is>
-          <t>Despesas e Custos</t>
+          <t>Investimentos Bens Imóveis</t>
         </is>
       </c>
     </row>
     <row r="1572">
       <c r="A1572" s="2" t="n">
-        <v>46333</v>
+        <v>46332</v>
       </c>
       <c r="B1572" t="inlineStr">
         <is>
-          <t>Apt. SP. - Condomínio (01)</t>
+          <t>Película para RANGER XLT</t>
         </is>
       </c>
       <c r="C1572" s="3" t="n">
-        <v>-1429.33</v>
+        <v>-100</v>
       </c>
       <c r="D1572" t="inlineStr">
         <is>
-          <t>Condomínio</t>
+          <t>Automóvel/Manutenção</t>
         </is>
       </c>
       <c r="E1572" t="inlineStr">
         <is>
-          <t>Conta BB</t>
+          <t>Cartão BB VISA</t>
         </is>
       </c>
       <c r="F1572" t="inlineStr">
@@ -70210,17 +70200,17 @@
       </c>
       <c r="G1572" t="inlineStr">
         <is>
-          <t>IMÓVEIS</t>
+          <t>TRANSPORTE</t>
         </is>
       </c>
       <c r="H1572" t="inlineStr">
         <is>
-          <t>Contas da casa</t>
+          <t>Automóvel</t>
         </is>
       </c>
       <c r="I1572" t="inlineStr">
         <is>
-          <t>Despesas com imóveis</t>
+          <t>Despesas com Automóvel (Manutenção)</t>
         </is>
       </c>
       <c r="J1572" t="inlineStr">
@@ -70231,24 +70221,24 @@
     </row>
     <row r="1573">
       <c r="A1573" s="2" t="n">
-        <v>46334</v>
+        <v>46332</v>
       </c>
       <c r="B1573" t="inlineStr">
         <is>
-          <t>Sapato para ACMD</t>
+          <t>Filtro para a COIFA - CONSUL</t>
         </is>
       </c>
       <c r="C1573" s="3" t="n">
-        <v>-121.6</v>
+        <v>-138.27</v>
       </c>
       <c r="D1573" t="inlineStr">
         <is>
-          <t>Roupas e Calçados</t>
+          <t>Restauração e Manutenção</t>
         </is>
       </c>
       <c r="E1573" t="inlineStr">
         <is>
-          <t>Cartão BB VISA</t>
+          <t>Cartão BB ELO</t>
         </is>
       </c>
       <c r="F1573" t="inlineStr">
@@ -70258,12 +70248,17 @@
       </c>
       <c r="G1573" t="inlineStr">
         <is>
-          <t>FAMÍLIA</t>
+          <t>IMÓVEIS</t>
+        </is>
+      </c>
+      <c r="H1573" t="inlineStr">
+        <is>
+          <t>Manutenção e encargos</t>
         </is>
       </c>
       <c r="I1573" t="inlineStr">
         <is>
-          <t>Despesas com família</t>
+          <t>Despesas com imóveis</t>
         </is>
       </c>
       <c r="J1573" t="inlineStr">
@@ -70274,24 +70269,24 @@
     </row>
     <row r="1574">
       <c r="A1574" s="2" t="n">
-        <v>46334</v>
+        <v>46333</v>
       </c>
       <c r="B1574" t="inlineStr">
         <is>
-          <t>Pagamento do estorno da AIR CANADA (1 e 2) em 02.03.2026</t>
+          <t>Apt. SP. - Condomínio (01)</t>
         </is>
       </c>
       <c r="C1574" s="3" t="n">
-        <v>-540.29</v>
+        <v>-1429.33</v>
       </c>
       <c r="D1574" t="inlineStr">
         <is>
-          <t>VIAGENS/Passagens</t>
+          <t>Condomínio</t>
         </is>
       </c>
       <c r="E1574" t="inlineStr">
         <is>
-          <t>Cartão BB VISA</t>
+          <t>Conta BB</t>
         </is>
       </c>
       <c r="F1574" t="inlineStr">
@@ -70301,17 +70296,17 @@
       </c>
       <c r="G1574" t="inlineStr">
         <is>
-          <t>LAZER</t>
+          <t>IMÓVEIS</t>
         </is>
       </c>
       <c r="H1574" t="inlineStr">
         <is>
-          <t>VIAGENS</t>
+          <t>Contas da casa</t>
         </is>
       </c>
       <c r="I1574" t="inlineStr">
         <is>
-          <t>Despesas com lazer</t>
+          <t>Despesas com imóveis</t>
         </is>
       </c>
       <c r="J1574" t="inlineStr">
@@ -70326,15 +70321,15 @@
       </c>
       <c r="B1575" t="inlineStr">
         <is>
-          <t>Pousada Aldeola em Baixio / Bahia (estadia)</t>
+          <t>Pagamento do estorno da AIR CANADA (1 e 2) em 02.03.2026</t>
         </is>
       </c>
       <c r="C1575" s="3" t="n">
-        <v>-124.64</v>
+        <v>-540.29</v>
       </c>
       <c r="D1575" t="inlineStr">
         <is>
-          <t>VIAGENS/Estadia</t>
+          <t>VIAGENS/Passagens</t>
         </is>
       </c>
       <c r="E1575" t="inlineStr">
@@ -70370,24 +70365,24 @@
     </row>
     <row r="1576">
       <c r="A1576" s="2" t="n">
-        <v>46335</v>
+        <v>46334</v>
       </c>
       <c r="B1576" t="inlineStr">
         <is>
-          <t>Resgate Parcial BB Deb Inc CDI Pvt</t>
+          <t>Sapato para ACMD</t>
         </is>
       </c>
       <c r="C1576" s="3" t="n">
-        <v>300000</v>
+        <v>-121.6</v>
       </c>
       <c r="D1576" t="inlineStr">
         <is>
-          <t>Resgate de Investimento</t>
+          <t>Roupas e Calçados</t>
         </is>
       </c>
       <c r="E1576" t="inlineStr">
         <is>
-          <t>Conta BB</t>
+          <t>Cartão BB VISA</t>
         </is>
       </c>
       <c r="F1576" t="inlineStr">
@@ -70397,40 +70392,40 @@
       </c>
       <c r="G1576" t="inlineStr">
         <is>
-          <t>INVESTIMENTOS E PATRIMÔNIO</t>
+          <t>FAMÍLIA</t>
         </is>
       </c>
       <c r="I1576" t="inlineStr">
         <is>
-          <t>Receitas Financeiras</t>
+          <t>Despesas com família</t>
         </is>
       </c>
       <c r="J1576" t="inlineStr">
         <is>
-          <t>Receitas Financeiras</t>
+          <t>Despesas e Custos</t>
         </is>
       </c>
     </row>
     <row r="1577">
       <c r="A1577" s="2" t="n">
-        <v>46336</v>
+        <v>46334</v>
       </c>
       <c r="B1577" t="inlineStr">
         <is>
-          <t>Aplicação Investimento Financeiro - BB RF REF DI Pvt</t>
+          <t>Pousada Aldeola em Baixio / Bahia (estadia)</t>
         </is>
       </c>
       <c r="C1577" s="3" t="n">
-        <v>-300000</v>
+        <v>-124.64</v>
       </c>
       <c r="D1577" t="inlineStr">
         <is>
-          <t>Aplicação em Investimento</t>
+          <t>VIAGENS/Estadia</t>
         </is>
       </c>
       <c r="E1577" t="inlineStr">
         <is>
-          <t>Conta BB</t>
+          <t>Cartão BB VISA</t>
         </is>
       </c>
       <c r="F1577" t="inlineStr">
@@ -70440,35 +70435,40 @@
       </c>
       <c r="G1577" t="inlineStr">
         <is>
-          <t>INVESTIMENTOS E PATRIMÔNIO</t>
+          <t>LAZER</t>
+        </is>
+      </c>
+      <c r="H1577" t="inlineStr">
+        <is>
+          <t>VIAGENS</t>
         </is>
       </c>
       <c r="I1577" t="inlineStr">
         <is>
-          <t>Investimentos Financeiros</t>
+          <t>Despesas com lazer</t>
         </is>
       </c>
       <c r="J1577" t="inlineStr">
         <is>
-          <t>Investimentos Financeiros</t>
+          <t>Despesas e Custos</t>
         </is>
       </c>
     </row>
     <row r="1578">
       <c r="A1578" s="2" t="n">
-        <v>46336</v>
+        <v>46335</v>
       </c>
       <c r="B1578" t="inlineStr">
         <is>
-          <t>Mensalidade da hidroginástica (10 / 11)</t>
+          <t>Resgate Parcial BB Deb Inc CDI Pvt</t>
         </is>
       </c>
       <c r="C1578" s="3" t="n">
-        <v>-88</v>
+        <v>300000</v>
       </c>
       <c r="D1578" t="inlineStr">
         <is>
-          <t>Academia</t>
+          <t>Resgate de Investimento</t>
         </is>
       </c>
       <c r="E1578" t="inlineStr">
@@ -70483,17 +70483,17 @@
       </c>
       <c r="G1578" t="inlineStr">
         <is>
-          <t>FAMÍLIA</t>
+          <t>INVESTIMENTOS E PATRIMÔNIO</t>
         </is>
       </c>
       <c r="I1578" t="inlineStr">
         <is>
-          <t>Despesas com família</t>
+          <t>Receitas Financeiras</t>
         </is>
       </c>
       <c r="J1578" t="inlineStr">
         <is>
-          <t>Despesas e Custos</t>
+          <t>Receitas Financeiras</t>
         </is>
       </c>
     </row>
@@ -70503,15 +70503,15 @@
       </c>
       <c r="B1579" t="inlineStr">
         <is>
-          <t>Plano OSAF - Serviços Funerários</t>
+          <t>Aplicação Investimento Financeiro - BB RF REF DI Pvt</t>
         </is>
       </c>
       <c r="C1579" s="3" t="n">
-        <v>-82.64</v>
+        <v>-300000</v>
       </c>
       <c r="D1579" t="inlineStr">
         <is>
-          <t>Serviços Funerários</t>
+          <t>Aplicação em Investimento</t>
         </is>
       </c>
       <c r="E1579" t="inlineStr">
@@ -70526,17 +70526,17 @@
       </c>
       <c r="G1579" t="inlineStr">
         <is>
-          <t>SEGUROS E SERVIÇOS FUNERÁRIOS</t>
+          <t>INVESTIMENTOS E PATRIMÔNIO</t>
         </is>
       </c>
       <c r="I1579" t="inlineStr">
         <is>
-          <t>Despesas com Seguros</t>
+          <t>Investimentos Financeiros</t>
         </is>
       </c>
       <c r="J1579" t="inlineStr">
         <is>
-          <t>Despesas e Custos</t>
+          <t>Investimentos Financeiros</t>
         </is>
       </c>
     </row>
@@ -70546,15 +70546,15 @@
       </c>
       <c r="B1580" t="inlineStr">
         <is>
-          <t>Hotel Stela Maris - Salvador</t>
+          <t>Mensalidade da hidroginástica (10 / 11)</t>
         </is>
       </c>
       <c r="C1580" s="3" t="n">
-        <v>-69.37</v>
+        <v>-88</v>
       </c>
       <c r="D1580" t="inlineStr">
         <is>
-          <t>VIAGENS/Estadia</t>
+          <t>Academia</t>
         </is>
       </c>
       <c r="E1580" t="inlineStr">
@@ -70569,17 +70569,12 @@
       </c>
       <c r="G1580" t="inlineStr">
         <is>
-          <t>LAZER</t>
-        </is>
-      </c>
-      <c r="H1580" t="inlineStr">
-        <is>
-          <t>VIAGENS</t>
+          <t>FAMÍLIA</t>
         </is>
       </c>
       <c r="I1580" t="inlineStr">
         <is>
-          <t>Despesas com lazer</t>
+          <t>Despesas com família</t>
         </is>
       </c>
       <c r="J1580" t="inlineStr">
@@ -70594,15 +70589,15 @@
       </c>
       <c r="B1581" t="inlineStr">
         <is>
-          <t>Aplicação PGBL BRASILPREV - ACMD</t>
+          <t>Plano OSAF - Serviços Funerários</t>
         </is>
       </c>
       <c r="C1581" s="3" t="n">
-        <v>-209.34</v>
+        <v>-82.64</v>
       </c>
       <c r="D1581" t="inlineStr">
         <is>
-          <t>BRASILPREV</t>
+          <t>Serviços Funerários</t>
         </is>
       </c>
       <c r="E1581" t="inlineStr">
@@ -70617,17 +70612,17 @@
       </c>
       <c r="G1581" t="inlineStr">
         <is>
-          <t>INVESTIMENTOS E PATRIMÔNIO</t>
+          <t>SEGUROS E SERVIÇOS FUNERÁRIOS</t>
         </is>
       </c>
       <c r="I1581" t="inlineStr">
         <is>
-          <t>Investimentos Financeiros</t>
+          <t>Despesas com Seguros</t>
         </is>
       </c>
       <c r="J1581" t="inlineStr">
         <is>
-          <t>Investimentos Financeiros</t>
+          <t>Despesas e Custos</t>
         </is>
       </c>
     </row>
@@ -70637,15 +70632,15 @@
       </c>
       <c r="B1582" t="inlineStr">
         <is>
-          <t>Presentes comprados por Gracinha (2026.10.14)</t>
+          <t>Hotel Stela Maris - Salvador</t>
         </is>
       </c>
       <c r="C1582" s="3" t="n">
-        <v>-134.38</v>
+        <v>-69.37</v>
       </c>
       <c r="D1582" t="inlineStr">
         <is>
-          <t>Presentes</t>
+          <t>VIAGENS/Estadia</t>
         </is>
       </c>
       <c r="E1582" t="inlineStr">
@@ -70660,12 +70655,17 @@
       </c>
       <c r="G1582" t="inlineStr">
         <is>
-          <t>FAMÍLIA</t>
+          <t>LAZER</t>
+        </is>
+      </c>
+      <c r="H1582" t="inlineStr">
+        <is>
+          <t>VIAGENS</t>
         </is>
       </c>
       <c r="I1582" t="inlineStr">
         <is>
-          <t>Despesas com família</t>
+          <t>Despesas com lazer</t>
         </is>
       </c>
       <c r="J1582" t="inlineStr">
@@ -70680,15 +70680,15 @@
       </c>
       <c r="B1583" t="inlineStr">
         <is>
-          <t>Casa Aracaju - Condomínio</t>
+          <t>Aplicação PGBL BRASILPREV - ACMD</t>
         </is>
       </c>
       <c r="C1583" s="3" t="n">
-        <v>-1650</v>
+        <v>-209.34</v>
       </c>
       <c r="D1583" t="inlineStr">
         <is>
-          <t>Condomínio</t>
+          <t>BRASILPREV</t>
         </is>
       </c>
       <c r="E1583" t="inlineStr">
@@ -70703,22 +70703,17 @@
       </c>
       <c r="G1583" t="inlineStr">
         <is>
-          <t>IMÓVEIS</t>
-        </is>
-      </c>
-      <c r="H1583" t="inlineStr">
-        <is>
-          <t>Contas da casa</t>
+          <t>INVESTIMENTOS E PATRIMÔNIO</t>
         </is>
       </c>
       <c r="I1583" t="inlineStr">
         <is>
-          <t>Despesas com imóveis</t>
+          <t>Investimentos Financeiros</t>
         </is>
       </c>
       <c r="J1583" t="inlineStr">
         <is>
-          <t>Despesas e Custos</t>
+          <t>Investimentos Financeiros</t>
         </is>
       </c>
     </row>
@@ -70728,15 +70723,15 @@
       </c>
       <c r="B1584" t="inlineStr">
         <is>
-          <t>Casa Aracaju - Taxa Extra (9 de 12 )</t>
+          <t>Presentes comprados por Gracinha (2026.10.14)</t>
         </is>
       </c>
       <c r="C1584" s="3" t="n">
-        <v>-500</v>
+        <v>-134.38</v>
       </c>
       <c r="D1584" t="inlineStr">
         <is>
-          <t>Ampliação-Melhorias Imóveis</t>
+          <t>Presentes</t>
         </is>
       </c>
       <c r="E1584" t="inlineStr">
@@ -70751,40 +70746,40 @@
       </c>
       <c r="G1584" t="inlineStr">
         <is>
-          <t>BENS DURÁVEIS</t>
+          <t>FAMÍLIA</t>
         </is>
       </c>
       <c r="I1584" t="inlineStr">
         <is>
-          <t>Investimentos Bens Imóveis</t>
+          <t>Despesas com família</t>
         </is>
       </c>
       <c r="J1584" t="inlineStr">
         <is>
-          <t>Investimentos Bens Imóveis</t>
+          <t>Despesas e Custos</t>
         </is>
       </c>
     </row>
     <row r="1585">
       <c r="A1585" s="2" t="n">
-        <v>46337</v>
+        <v>46336</v>
       </c>
       <c r="B1585" t="inlineStr">
         <is>
-          <t>Casa Aracaju - Toldo de proteção para a garagem</t>
+          <t>Casa Aracaju - Condomínio</t>
         </is>
       </c>
       <c r="C1585" s="3" t="n">
-        <v>-1818.04</v>
+        <v>-1650</v>
       </c>
       <c r="D1585" t="inlineStr">
         <is>
-          <t>Ampliação-Melhorias Imóveis</t>
+          <t>Condomínio</t>
         </is>
       </c>
       <c r="E1585" t="inlineStr">
         <is>
-          <t>Cartão BB VISA</t>
+          <t>Conta BB</t>
         </is>
       </c>
       <c r="F1585" t="inlineStr">
@@ -70794,40 +70789,45 @@
       </c>
       <c r="G1585" t="inlineStr">
         <is>
-          <t>BENS DURÁVEIS</t>
+          <t>IMÓVEIS</t>
+        </is>
+      </c>
+      <c r="H1585" t="inlineStr">
+        <is>
+          <t>Contas da casa</t>
         </is>
       </c>
       <c r="I1585" t="inlineStr">
         <is>
-          <t>Investimentos Bens Imóveis</t>
+          <t>Despesas com imóveis</t>
         </is>
       </c>
       <c r="J1585" t="inlineStr">
         <is>
-          <t>Investimentos Bens Imóveis</t>
+          <t>Despesas e Custos</t>
         </is>
       </c>
     </row>
     <row r="1586">
       <c r="A1586" s="2" t="n">
-        <v>46338</v>
+        <v>46336</v>
       </c>
       <c r="B1586" t="inlineStr">
         <is>
-          <t>Aluguel do terno para o casamento de João Paulo</t>
+          <t>Casa Aracaju - Taxa Extra (9 de 12 )</t>
         </is>
       </c>
       <c r="C1586" s="3" t="n">
-        <v>-116.67</v>
+        <v>-500</v>
       </c>
       <c r="D1586" t="inlineStr">
         <is>
-          <t>Roupas e Calçados</t>
+          <t>Ampliação-Melhorias Imóveis</t>
         </is>
       </c>
       <c r="E1586" t="inlineStr">
         <is>
-          <t>Cartão BB VISA</t>
+          <t>Conta BB</t>
         </is>
       </c>
       <c r="F1586" t="inlineStr">
@@ -70837,35 +70837,35 @@
       </c>
       <c r="G1586" t="inlineStr">
         <is>
-          <t>FAMÍLIA</t>
+          <t>BENS DURÁVEIS</t>
         </is>
       </c>
       <c r="I1586" t="inlineStr">
         <is>
-          <t>Despesas com família</t>
+          <t>Investimentos Bens Imóveis</t>
         </is>
       </c>
       <c r="J1586" t="inlineStr">
         <is>
-          <t>Despesas e Custos</t>
+          <t>Investimentos Bens Imóveis</t>
         </is>
       </c>
     </row>
     <row r="1587">
       <c r="A1587" s="2" t="n">
-        <v>46339</v>
+        <v>46337</v>
       </c>
       <c r="B1587" t="inlineStr">
         <is>
-          <t>Casa Aracaju - Cabo PP para interligar o carregador de Bateria do BYD</t>
+          <t>Casa Aracaju - Toldo de proteção para a garagem</t>
         </is>
       </c>
       <c r="C1587" s="3" t="n">
-        <v>-58.07</v>
+        <v>-1818.04</v>
       </c>
       <c r="D1587" t="inlineStr">
         <is>
-          <t>Eletrônicos</t>
+          <t>Ampliação-Melhorias Imóveis</t>
         </is>
       </c>
       <c r="E1587" t="inlineStr">
@@ -70885,30 +70885,30 @@
       </c>
       <c r="I1587" t="inlineStr">
         <is>
-          <t>Investimentos Bens</t>
+          <t>Investimentos Bens Imóveis</t>
         </is>
       </c>
       <c r="J1587" t="inlineStr">
         <is>
-          <t>Investimentos</t>
+          <t>Investimentos Bens Imóveis</t>
         </is>
       </c>
     </row>
     <row r="1588">
       <c r="A1588" s="2" t="n">
-        <v>46339</v>
+        <v>46338</v>
       </c>
       <c r="B1588" t="inlineStr">
         <is>
-          <t>Seguro da Hilux SW4</t>
+          <t>Aluguel do terno para o casamento de João Paulo</t>
         </is>
       </c>
       <c r="C1588" s="3" t="n">
-        <v>-233.11</v>
+        <v>-116.67</v>
       </c>
       <c r="D1588" t="inlineStr">
         <is>
-          <t>Automóvel/Seguro</t>
+          <t>Roupas e Calçados</t>
         </is>
       </c>
       <c r="E1588" t="inlineStr">
@@ -70923,17 +70923,12 @@
       </c>
       <c r="G1588" t="inlineStr">
         <is>
-          <t>TRANSPORTE</t>
-        </is>
-      </c>
-      <c r="H1588" t="inlineStr">
-        <is>
-          <t>Automóvel</t>
+          <t>FAMÍLIA</t>
         </is>
       </c>
       <c r="I1588" t="inlineStr">
         <is>
-          <t>Despesas com Automóvel (Seguros)</t>
+          <t>Despesas com família</t>
         </is>
       </c>
       <c r="J1588" t="inlineStr">
@@ -70992,19 +70987,19 @@
     </row>
     <row r="1590">
       <c r="A1590" s="2" t="n">
-        <v>46341</v>
+        <v>46339</v>
       </c>
       <c r="B1590" t="inlineStr">
         <is>
-          <t>Remédios para ACMD</t>
+          <t>Seguro da Hilux SW4</t>
         </is>
       </c>
       <c r="C1590" s="3" t="n">
-        <v>-52.83</v>
+        <v>-233.11</v>
       </c>
       <c r="D1590" t="inlineStr">
         <is>
-          <t>Farmácia</t>
+          <t>Automóvel/Seguro</t>
         </is>
       </c>
       <c r="E1590" t="inlineStr">
@@ -71019,12 +71014,17 @@
       </c>
       <c r="G1590" t="inlineStr">
         <is>
-          <t>SAÚDE</t>
+          <t>TRANSPORTE</t>
+        </is>
+      </c>
+      <c r="H1590" t="inlineStr">
+        <is>
+          <t>Automóvel</t>
         </is>
       </c>
       <c r="I1590" t="inlineStr">
         <is>
-          <t>Despesas com Saúde</t>
+          <t>Despesas com Automóvel (Seguros)</t>
         </is>
       </c>
       <c r="J1590" t="inlineStr">
@@ -71035,19 +71035,19 @@
     </row>
     <row r="1591">
       <c r="A1591" s="2" t="n">
-        <v>46341</v>
+        <v>46339</v>
       </c>
       <c r="B1591" t="inlineStr">
         <is>
-          <t>Pagamento Clube SMILES</t>
+          <t>Casa Aracaju - Cabo PP para interligar o carregador de Bateria do BYD</t>
         </is>
       </c>
       <c r="C1591" s="3" t="n">
-        <v>-46</v>
+        <v>-58.07</v>
       </c>
       <c r="D1591" t="inlineStr">
         <is>
-          <t>VIAGENS/Passagens</t>
+          <t>Eletrônicos</t>
         </is>
       </c>
       <c r="E1591" t="inlineStr">
@@ -71062,40 +71062,35 @@
       </c>
       <c r="G1591" t="inlineStr">
         <is>
-          <t>LAZER</t>
-        </is>
-      </c>
-      <c r="H1591" t="inlineStr">
-        <is>
-          <t>VIAGENS</t>
+          <t>BENS DURÁVEIS</t>
         </is>
       </c>
       <c r="I1591" t="inlineStr">
         <is>
-          <t>Despesas com lazer</t>
+          <t>Investimentos Bens</t>
         </is>
       </c>
       <c r="J1591" t="inlineStr">
         <is>
-          <t>Despesas e Custos</t>
+          <t>Investimentos</t>
         </is>
       </c>
     </row>
     <row r="1592">
       <c r="A1592" s="2" t="n">
-        <v>46342</v>
+        <v>46341</v>
       </c>
       <c r="B1592" t="inlineStr">
         <is>
-          <t>Transporte Terrestre, Hoteis e Excursão</t>
+          <t>Remédios para ACMD</t>
         </is>
       </c>
       <c r="C1592" s="3" t="n">
-        <v>-1824.26</v>
+        <v>-52.83</v>
       </c>
       <c r="D1592" t="inlineStr">
         <is>
-          <t>VIAGENS/Passeios</t>
+          <t>Farmácia</t>
         </is>
       </c>
       <c r="E1592" t="inlineStr">
@@ -71110,17 +71105,12 @@
       </c>
       <c r="G1592" t="inlineStr">
         <is>
-          <t>LAZER</t>
-        </is>
-      </c>
-      <c r="H1592" t="inlineStr">
-        <is>
-          <t>VIAGENS</t>
+          <t>SAÚDE</t>
         </is>
       </c>
       <c r="I1592" t="inlineStr">
         <is>
-          <t>Despesas com lazer</t>
+          <t>Despesas com Saúde</t>
         </is>
       </c>
       <c r="J1592" t="inlineStr">
@@ -71131,19 +71121,19 @@
     </row>
     <row r="1593">
       <c r="A1593" s="2" t="n">
-        <v>46342</v>
+        <v>46341</v>
       </c>
       <c r="B1593" t="inlineStr">
         <is>
-          <t>Academia ACMD</t>
+          <t>Pagamento Clube SMILES</t>
         </is>
       </c>
       <c r="C1593" s="3" t="n">
-        <v>-448.35</v>
+        <v>-46</v>
       </c>
       <c r="D1593" t="inlineStr">
         <is>
-          <t>Academia</t>
+          <t>VIAGENS/Passagens</t>
         </is>
       </c>
       <c r="E1593" t="inlineStr">
@@ -71158,12 +71148,17 @@
       </c>
       <c r="G1593" t="inlineStr">
         <is>
-          <t>FAMÍLIA</t>
+          <t>LAZER</t>
+        </is>
+      </c>
+      <c r="H1593" t="inlineStr">
+        <is>
+          <t>VIAGENS</t>
         </is>
       </c>
       <c r="I1593" t="inlineStr">
         <is>
-          <t>Despesas com família</t>
+          <t>Despesas com lazer</t>
         </is>
       </c>
       <c r="J1593" t="inlineStr">
@@ -71174,19 +71169,19 @@
     </row>
     <row r="1594">
       <c r="A1594" s="2" t="n">
-        <v>46345</v>
+        <v>46342</v>
       </c>
       <c r="B1594" t="inlineStr">
         <is>
-          <t>Perfume no Boticário</t>
+          <t>Academia ACMD</t>
         </is>
       </c>
       <c r="C1594" s="3" t="n">
-        <v>-8.99</v>
+        <v>-448.35</v>
       </c>
       <c r="D1594" t="inlineStr">
         <is>
-          <t>Salão de Beleza e Cosméticos</t>
+          <t>Academia</t>
         </is>
       </c>
       <c r="E1594" t="inlineStr">
@@ -71217,19 +71212,19 @@
     </row>
     <row r="1595">
       <c r="A1595" s="2" t="n">
-        <v>46346</v>
+        <v>46342</v>
       </c>
       <c r="B1595" t="inlineStr">
         <is>
-          <t>Sacos para os alimentos dos necessitados (2 / 2)</t>
+          <t>Transporte Terrestre, Hoteis e Excursão</t>
         </is>
       </c>
       <c r="C1595" s="3" t="n">
-        <v>-72</v>
+        <v>-1824.26</v>
       </c>
       <c r="D1595" t="inlineStr">
         <is>
-          <t>Feira e Mercearia</t>
+          <t>VIAGENS/Passeios</t>
         </is>
       </c>
       <c r="E1595" t="inlineStr">
@@ -71244,12 +71239,17 @@
       </c>
       <c r="G1595" t="inlineStr">
         <is>
-          <t>ALIMENTAÇÃO E LIMPEZA</t>
+          <t>LAZER</t>
+        </is>
+      </c>
+      <c r="H1595" t="inlineStr">
+        <is>
+          <t>VIAGENS</t>
         </is>
       </c>
       <c r="I1595" t="inlineStr">
         <is>
-          <t>Despesas com alimentação e limpeza</t>
+          <t>Despesas com lazer</t>
         </is>
       </c>
       <c r="J1595" t="inlineStr">
@@ -71260,19 +71260,19 @@
     </row>
     <row r="1596">
       <c r="A1596" s="2" t="n">
-        <v>46346</v>
+        <v>46345</v>
       </c>
       <c r="B1596" t="inlineStr">
         <is>
-          <t>Materiais de limpeza (2 / 2)</t>
+          <t>Perfume no Boticário</t>
         </is>
       </c>
       <c r="C1596" s="3" t="n">
-        <v>-110.2</v>
+        <v>-8.99</v>
       </c>
       <c r="D1596" t="inlineStr">
         <is>
-          <t>Feira e Mercearia</t>
+          <t>Salão de Beleza e Cosméticos</t>
         </is>
       </c>
       <c r="E1596" t="inlineStr">
@@ -71287,12 +71287,12 @@
       </c>
       <c r="G1596" t="inlineStr">
         <is>
-          <t>ALIMENTAÇÃO E LIMPEZA</t>
+          <t>FAMÍLIA</t>
         </is>
       </c>
       <c r="I1596" t="inlineStr">
         <is>
-          <t>Despesas com alimentação e limpeza</t>
+          <t>Despesas com família</t>
         </is>
       </c>
       <c r="J1596" t="inlineStr">
@@ -71303,19 +71303,19 @@
     </row>
     <row r="1597">
       <c r="A1597" s="2" t="n">
-        <v>46347</v>
+        <v>46346</v>
       </c>
       <c r="B1597" t="inlineStr">
         <is>
-          <t>Aluguel de terno para Nicholas (2 / 2)</t>
+          <t>Sacos para os alimentos dos necessitados (2 / 2)</t>
         </is>
       </c>
       <c r="C1597" s="3" t="n">
-        <v>-175</v>
+        <v>-72</v>
       </c>
       <c r="D1597" t="inlineStr">
         <is>
-          <t>Roupas e Calçados</t>
+          <t>Feira e Mercearia</t>
         </is>
       </c>
       <c r="E1597" t="inlineStr">
@@ -71330,12 +71330,12 @@
       </c>
       <c r="G1597" t="inlineStr">
         <is>
-          <t>FAMÍLIA</t>
+          <t>ALIMENTAÇÃO E LIMPEZA</t>
         </is>
       </c>
       <c r="I1597" t="inlineStr">
         <is>
-          <t>Despesas com família</t>
+          <t>Despesas com alimentação e limpeza</t>
         </is>
       </c>
       <c r="J1597" t="inlineStr">
@@ -71346,24 +71346,24 @@
     </row>
     <row r="1598">
       <c r="A1598" s="2" t="n">
-        <v>46347</v>
+        <v>46346</v>
       </c>
       <c r="B1598" t="inlineStr">
         <is>
-          <t>Apt. SP. - Condomínio (02)</t>
+          <t>Materiais de limpeza (2 / 2)</t>
         </is>
       </c>
       <c r="C1598" s="3" t="n">
-        <v>-1063.47</v>
+        <v>-110.2</v>
       </c>
       <c r="D1598" t="inlineStr">
         <is>
-          <t>Condomínio</t>
+          <t>Feira e Mercearia</t>
         </is>
       </c>
       <c r="E1598" t="inlineStr">
         <is>
-          <t>Conta BB</t>
+          <t>Cartão BB VISA</t>
         </is>
       </c>
       <c r="F1598" t="inlineStr">
@@ -71373,17 +71373,12 @@
       </c>
       <c r="G1598" t="inlineStr">
         <is>
-          <t>IMÓVEIS</t>
-        </is>
-      </c>
-      <c r="H1598" t="inlineStr">
-        <is>
-          <t>Contas da casa</t>
+          <t>ALIMENTAÇÃO E LIMPEZA</t>
         </is>
       </c>
       <c r="I1598" t="inlineStr">
         <is>
-          <t>Despesas com imóveis</t>
+          <t>Despesas com alimentação e limpeza</t>
         </is>
       </c>
       <c r="J1598" t="inlineStr">
@@ -71394,24 +71389,24 @@
     </row>
     <row r="1599">
       <c r="A1599" s="2" t="n">
-        <v>46348</v>
+        <v>46347</v>
       </c>
       <c r="B1599" t="inlineStr">
         <is>
-          <t>Lata de lixo e outros utensílios domésticos</t>
+          <t>Apt. SP. - Condomínio (02)</t>
         </is>
       </c>
       <c r="C1599" s="3" t="n">
-        <v>-53.66</v>
+        <v>-1063.47</v>
       </c>
       <c r="D1599" t="inlineStr">
         <is>
-          <t>Restauração e Manutenção</t>
+          <t>Condomínio</t>
         </is>
       </c>
       <c r="E1599" t="inlineStr">
         <is>
-          <t>Cartão BB VISA</t>
+          <t>Conta BB</t>
         </is>
       </c>
       <c r="F1599" t="inlineStr">
@@ -71426,7 +71421,7 @@
       </c>
       <c r="H1599" t="inlineStr">
         <is>
-          <t>Manutenção e encargos</t>
+          <t>Contas da casa</t>
         </is>
       </c>
       <c r="I1599" t="inlineStr">
@@ -71442,19 +71437,19 @@
     </row>
     <row r="1600">
       <c r="A1600" s="2" t="n">
-        <v>46348</v>
+        <v>46347</v>
       </c>
       <c r="B1600" t="inlineStr">
         <is>
-          <t>Casa Aracaju - Materiais para o jardim</t>
+          <t>Aluguel de terno para Nicholas (2 / 2)</t>
         </is>
       </c>
       <c r="C1600" s="3" t="n">
-        <v>-112.07</v>
+        <v>-175</v>
       </c>
       <c r="D1600" t="inlineStr">
         <is>
-          <t>Restauração e Manutenção</t>
+          <t>Roupas e Calçados</t>
         </is>
       </c>
       <c r="E1600" t="inlineStr">
@@ -71469,17 +71464,12 @@
       </c>
       <c r="G1600" t="inlineStr">
         <is>
-          <t>IMÓVEIS</t>
-        </is>
-      </c>
-      <c r="H1600" t="inlineStr">
-        <is>
-          <t>Manutenção e encargos</t>
+          <t>FAMÍLIA</t>
         </is>
       </c>
       <c r="I1600" t="inlineStr">
         <is>
-          <t>Despesas com imóveis</t>
+          <t>Despesas com família</t>
         </is>
       </c>
       <c r="J1600" t="inlineStr">
@@ -71490,19 +71480,19 @@
     </row>
     <row r="1601">
       <c r="A1601" s="2" t="n">
-        <v>46350</v>
+        <v>46348</v>
       </c>
       <c r="B1601" t="inlineStr">
         <is>
-          <t>Instalação das câmeras lateral e frontal na RANGER xLT</t>
+          <t>Lata de lixo e outros utensílios domésticos</t>
         </is>
       </c>
       <c r="C1601" s="3" t="n">
-        <v>-500</v>
+        <v>-53.66</v>
       </c>
       <c r="D1601" t="inlineStr">
         <is>
-          <t>Automóvel/Manutenção</t>
+          <t>Restauração e Manutenção</t>
         </is>
       </c>
       <c r="E1601" t="inlineStr">
@@ -71517,17 +71507,17 @@
       </c>
       <c r="G1601" t="inlineStr">
         <is>
-          <t>TRANSPORTE</t>
+          <t>IMÓVEIS</t>
         </is>
       </c>
       <c r="H1601" t="inlineStr">
         <is>
-          <t>Automóvel</t>
+          <t>Manutenção e encargos</t>
         </is>
       </c>
       <c r="I1601" t="inlineStr">
         <is>
-          <t>Despesas com Automóvel (Manutenção)</t>
+          <t>Despesas com imóveis</t>
         </is>
       </c>
       <c r="J1601" t="inlineStr">
@@ -71538,24 +71528,24 @@
     </row>
     <row r="1602">
       <c r="A1602" s="2" t="n">
-        <v>46351</v>
+        <v>46348</v>
       </c>
       <c r="B1602" t="inlineStr">
         <is>
-          <t>Pagamento "DUO GOURMET"</t>
+          <t>Casa Aracaju - Materiais para o jardim</t>
         </is>
       </c>
       <c r="C1602" s="3" t="n">
-        <v>-45</v>
+        <v>-112.07</v>
       </c>
       <c r="D1602" t="inlineStr">
         <is>
-          <t>Restaurante</t>
+          <t>Restauração e Manutenção</t>
         </is>
       </c>
       <c r="E1602" t="inlineStr">
         <is>
-          <t>Conta BB</t>
+          <t>Cartão BB VISA</t>
         </is>
       </c>
       <c r="F1602" t="inlineStr">
@@ -71565,12 +71555,17 @@
       </c>
       <c r="G1602" t="inlineStr">
         <is>
-          <t>ALIMENTAÇÃO E LIMPEZA</t>
+          <t>IMÓVEIS</t>
+        </is>
+      </c>
+      <c r="H1602" t="inlineStr">
+        <is>
+          <t>Manutenção e encargos</t>
         </is>
       </c>
       <c r="I1602" t="inlineStr">
         <is>
-          <t>Despesas com alimentação e limpeza</t>
+          <t>Despesas com imóveis</t>
         </is>
       </c>
       <c r="J1602" t="inlineStr">
@@ -71581,19 +71576,19 @@
     </row>
     <row r="1603">
       <c r="A1603" s="2" t="n">
-        <v>46353</v>
+        <v>46350</v>
       </c>
       <c r="B1603" t="inlineStr">
         <is>
-          <t>Troca da bateria do MACBOOK PRO</t>
+          <t>Instalação das câmeras lateral e frontal na RANGER xLT</t>
         </is>
       </c>
       <c r="C1603" s="3" t="n">
-        <v>-102.5</v>
+        <v>-500</v>
       </c>
       <c r="D1603" t="inlineStr">
         <is>
-          <t>OUTRAS DESPESAS</t>
+          <t>Automóvel/Manutenção</t>
         </is>
       </c>
       <c r="E1603" t="inlineStr">
@@ -71608,12 +71603,17 @@
       </c>
       <c r="G1603" t="inlineStr">
         <is>
-          <t>OUTRAS DESPESAS</t>
+          <t>TRANSPORTE</t>
+        </is>
+      </c>
+      <c r="H1603" t="inlineStr">
+        <is>
+          <t>Automóvel</t>
         </is>
       </c>
       <c r="I1603" t="inlineStr">
         <is>
-          <t>Outras Despesas</t>
+          <t>Despesas com Automóvel (Manutenção)</t>
         </is>
       </c>
       <c r="J1603" t="inlineStr">
@@ -71624,24 +71624,24 @@
     </row>
     <row r="1604">
       <c r="A1604" s="2" t="n">
-        <v>46353</v>
+        <v>46351</v>
       </c>
       <c r="B1604" t="inlineStr">
         <is>
-          <t>Aquisição do celular MOTOROLA G86</t>
+          <t>Pagamento "DUO GOURMET"</t>
         </is>
       </c>
       <c r="C1604" s="3" t="n">
-        <v>-139</v>
+        <v>-45</v>
       </c>
       <c r="D1604" t="inlineStr">
         <is>
-          <t>Eletrônicos</t>
+          <t>Restaurante</t>
         </is>
       </c>
       <c r="E1604" t="inlineStr">
         <is>
-          <t>Cartão BB VISA</t>
+          <t>Conta BB</t>
         </is>
       </c>
       <c r="F1604" t="inlineStr">
@@ -71651,35 +71651,35 @@
       </c>
       <c r="G1604" t="inlineStr">
         <is>
-          <t>BENS DURÁVEIS</t>
+          <t>ALIMENTAÇÃO E LIMPEZA</t>
         </is>
       </c>
       <c r="I1604" t="inlineStr">
         <is>
-          <t>Investimentos Bens</t>
+          <t>Despesas com alimentação e limpeza</t>
         </is>
       </c>
       <c r="J1604" t="inlineStr">
         <is>
-          <t>Investimentos</t>
+          <t>Despesas e Custos</t>
         </is>
       </c>
     </row>
     <row r="1605">
       <c r="A1605" s="2" t="n">
-        <v>46354</v>
+        <v>46353</v>
       </c>
       <c r="B1605" t="inlineStr">
         <is>
-          <t>TV SAMSUNG quarto do casal (7 / 8)</t>
+          <t>Aquisição do celular MOTOROLA G86</t>
         </is>
       </c>
       <c r="C1605" s="3" t="n">
-        <v>-337.49</v>
+        <v>-139</v>
       </c>
       <c r="D1605" t="inlineStr">
         <is>
-          <t>Acessórios</t>
+          <t>Eletrônicos</t>
         </is>
       </c>
       <c r="E1605" t="inlineStr">
@@ -71694,40 +71694,40 @@
       </c>
       <c r="G1605" t="inlineStr">
         <is>
-          <t>FAMÍLIA</t>
+          <t>BENS DURÁVEIS</t>
         </is>
       </c>
       <c r="I1605" t="inlineStr">
         <is>
-          <t>Despesas com família</t>
+          <t>Investimentos Bens</t>
         </is>
       </c>
       <c r="J1605" t="inlineStr">
         <is>
-          <t>Despesas e Custos</t>
+          <t>Investimentos</t>
         </is>
       </c>
     </row>
     <row r="1606">
       <c r="A1606" s="2" t="n">
-        <v>46357</v>
+        <v>46353</v>
       </c>
       <c r="B1606" t="inlineStr">
         <is>
-          <t>Seguro Apt Aracaju - Parcelas 4</t>
+          <t>Troca da bateria do MACBOOK PRO</t>
         </is>
       </c>
       <c r="C1606" s="3" t="n">
-        <v>-52.85</v>
+        <v>-102.5</v>
       </c>
       <c r="D1606" t="inlineStr">
         <is>
-          <t>Residencial</t>
+          <t>OUTRAS DESPESAS</t>
         </is>
       </c>
       <c r="E1606" t="inlineStr">
         <is>
-          <t>Conta BB</t>
+          <t>Cartão BB VISA</t>
         </is>
       </c>
       <c r="F1606" t="inlineStr">
@@ -71737,12 +71737,12 @@
       </c>
       <c r="G1606" t="inlineStr">
         <is>
-          <t>SEGUROS E SERVIÇOS FUNERÁRIOS</t>
+          <t>OUTRAS DESPESAS</t>
         </is>
       </c>
       <c r="I1606" t="inlineStr">
         <is>
-          <t>Despesas com Seguros</t>
+          <t>Outras Despesas</t>
         </is>
       </c>
       <c r="J1606" t="inlineStr">
@@ -71753,24 +71753,24 @@
     </row>
     <row r="1607">
       <c r="A1607" s="2" t="n">
-        <v>46358</v>
+        <v>46354</v>
       </c>
       <c r="B1607" t="inlineStr">
         <is>
-          <t>Seguro de Itens Pessoais</t>
+          <t>TV SAMSUNG quarto do casal (7 / 8)</t>
         </is>
       </c>
       <c r="C1607" s="3" t="n">
-        <v>-9.9</v>
+        <v>-337.49</v>
       </c>
       <c r="D1607" t="inlineStr">
         <is>
-          <t>Equipamentos Eletrônicos</t>
+          <t>Acessórios</t>
         </is>
       </c>
       <c r="E1607" t="inlineStr">
         <is>
-          <t>Conta BB</t>
+          <t>Cartão BB VISA</t>
         </is>
       </c>
       <c r="F1607" t="inlineStr">
@@ -71780,12 +71780,12 @@
       </c>
       <c r="G1607" t="inlineStr">
         <is>
-          <t>SEGUROS E SERVIÇOS FUNERÁRIOS</t>
+          <t>FAMÍLIA</t>
         </is>
       </c>
       <c r="I1607" t="inlineStr">
         <is>
-          <t>Despesas com Seguros</t>
+          <t>Despesas com família</t>
         </is>
       </c>
       <c r="J1607" t="inlineStr">
@@ -71796,19 +71796,19 @@
     </row>
     <row r="1608">
       <c r="A1608" s="2" t="n">
-        <v>46362</v>
+        <v>46357</v>
       </c>
       <c r="B1608" t="inlineStr">
         <is>
-          <t>Casa Aracaju - Aquisição e instalação da piscina</t>
+          <t>Seguro Apt Aracaju - Parcelas 4</t>
         </is>
       </c>
       <c r="C1608" s="3" t="n">
-        <v>-17600</v>
+        <v>-52.85</v>
       </c>
       <c r="D1608" t="inlineStr">
         <is>
-          <t>Ampliação-Melhorias Imóveis</t>
+          <t>Residencial</t>
         </is>
       </c>
       <c r="E1608" t="inlineStr">
@@ -71823,40 +71823,40 @@
       </c>
       <c r="G1608" t="inlineStr">
         <is>
-          <t>BENS DURÁVEIS</t>
+          <t>SEGUROS E SERVIÇOS FUNERÁRIOS</t>
         </is>
       </c>
       <c r="I1608" t="inlineStr">
         <is>
-          <t>Investimentos Bens Imóveis</t>
+          <t>Despesas com Seguros</t>
         </is>
       </c>
       <c r="J1608" t="inlineStr">
         <is>
-          <t>Investimentos Bens Imóveis</t>
+          <t>Despesas e Custos</t>
         </is>
       </c>
     </row>
     <row r="1609">
       <c r="A1609" s="2" t="n">
-        <v>46362</v>
+        <v>46358</v>
       </c>
       <c r="B1609" t="inlineStr">
         <is>
-          <t>Película para RANGER XLT</t>
+          <t>Seguro de Itens Pessoais</t>
         </is>
       </c>
       <c r="C1609" s="3" t="n">
-        <v>-100</v>
+        <v>-9.9</v>
       </c>
       <c r="D1609" t="inlineStr">
         <is>
-          <t>Automóvel/Manutenção</t>
+          <t>Equipamentos Eletrônicos</t>
         </is>
       </c>
       <c r="E1609" t="inlineStr">
         <is>
-          <t>Cartão BB VISA</t>
+          <t>Conta BB</t>
         </is>
       </c>
       <c r="F1609" t="inlineStr">
@@ -71866,17 +71866,12 @@
       </c>
       <c r="G1609" t="inlineStr">
         <is>
-          <t>TRANSPORTE</t>
-        </is>
-      </c>
-      <c r="H1609" t="inlineStr">
-        <is>
-          <t>Automóvel</t>
+          <t>SEGUROS E SERVIÇOS FUNERÁRIOS</t>
         </is>
       </c>
       <c r="I1609" t="inlineStr">
         <is>
-          <t>Despesas com Automóvel (Manutenção)</t>
+          <t>Despesas com Seguros</t>
         </is>
       </c>
       <c r="J1609" t="inlineStr">
@@ -71887,24 +71882,24 @@
     </row>
     <row r="1610">
       <c r="A1610" s="2" t="n">
-        <v>46364</v>
+        <v>46362</v>
       </c>
       <c r="B1610" t="inlineStr">
         <is>
-          <t>Pousada Aldeola em Baixio / Bahia (estadia)</t>
+          <t>Casa Aracaju - Aquisição e instalação da piscina</t>
         </is>
       </c>
       <c r="C1610" s="3" t="n">
-        <v>-124.64</v>
+        <v>-17600</v>
       </c>
       <c r="D1610" t="inlineStr">
         <is>
-          <t>VIAGENS/Estadia</t>
+          <t>Ampliação-Melhorias Imóveis</t>
         </is>
       </c>
       <c r="E1610" t="inlineStr">
         <is>
-          <t>Cartão BB VISA</t>
+          <t>Conta BB</t>
         </is>
       </c>
       <c r="F1610" t="inlineStr">
@@ -71914,40 +71909,35 @@
       </c>
       <c r="G1610" t="inlineStr">
         <is>
-          <t>LAZER</t>
-        </is>
-      </c>
-      <c r="H1610" t="inlineStr">
-        <is>
-          <t>VIAGENS</t>
+          <t>BENS DURÁVEIS</t>
         </is>
       </c>
       <c r="I1610" t="inlineStr">
         <is>
-          <t>Despesas com lazer</t>
+          <t>Investimentos Bens Imóveis</t>
         </is>
       </c>
       <c r="J1610" t="inlineStr">
         <is>
-          <t>Despesas e Custos</t>
+          <t>Investimentos Bens Imóveis</t>
         </is>
       </c>
     </row>
     <row r="1611">
       <c r="A1611" s="2" t="n">
-        <v>46364</v>
+        <v>46362</v>
       </c>
       <c r="B1611" t="inlineStr">
         <is>
-          <t>Pagamento do estorno da AIR CANADA (1 e 2) em 02.03.2026</t>
+          <t>Película para RANGER XLT</t>
         </is>
       </c>
       <c r="C1611" s="3" t="n">
-        <v>-540.29</v>
+        <v>-100</v>
       </c>
       <c r="D1611" t="inlineStr">
         <is>
-          <t>VIAGENS/Passagens</t>
+          <t>Automóvel/Manutenção</t>
         </is>
       </c>
       <c r="E1611" t="inlineStr">
@@ -71962,17 +71952,17 @@
       </c>
       <c r="G1611" t="inlineStr">
         <is>
-          <t>LAZER</t>
+          <t>TRANSPORTE</t>
         </is>
       </c>
       <c r="H1611" t="inlineStr">
         <is>
-          <t>VIAGENS</t>
+          <t>Automóvel</t>
         </is>
       </c>
       <c r="I1611" t="inlineStr">
         <is>
-          <t>Despesas com lazer</t>
+          <t>Despesas com Automóvel (Manutenção)</t>
         </is>
       </c>
       <c r="J1611" t="inlineStr">
@@ -71983,24 +71973,24 @@
     </row>
     <row r="1612">
       <c r="A1612" s="2" t="n">
-        <v>46366</v>
+        <v>46364</v>
       </c>
       <c r="B1612" t="inlineStr">
         <is>
-          <t>Mensalidade da hidroginástica (11 / 11)</t>
+          <t>Pousada Aldeola em Baixio / Bahia (estadia)</t>
         </is>
       </c>
       <c r="C1612" s="3" t="n">
-        <v>-23.46</v>
+        <v>-124.64</v>
       </c>
       <c r="D1612" t="inlineStr">
         <is>
-          <t>Academia</t>
+          <t>VIAGENS/Estadia</t>
         </is>
       </c>
       <c r="E1612" t="inlineStr">
         <is>
-          <t>Conta BB</t>
+          <t>Cartão BB VISA</t>
         </is>
       </c>
       <c r="F1612" t="inlineStr">
@@ -72010,12 +72000,17 @@
       </c>
       <c r="G1612" t="inlineStr">
         <is>
-          <t>FAMÍLIA</t>
+          <t>LAZER</t>
+        </is>
+      </c>
+      <c r="H1612" t="inlineStr">
+        <is>
+          <t>VIAGENS</t>
         </is>
       </c>
       <c r="I1612" t="inlineStr">
         <is>
-          <t>Despesas com família</t>
+          <t>Despesas com lazer</t>
         </is>
       </c>
       <c r="J1612" t="inlineStr">
@@ -72026,24 +72021,24 @@
     </row>
     <row r="1613">
       <c r="A1613" s="2" t="n">
-        <v>46366</v>
+        <v>46364</v>
       </c>
       <c r="B1613" t="inlineStr">
         <is>
-          <t>Plano OSAF - Serviços Funerários</t>
+          <t>Pagamento do estorno da AIR CANADA (1 e 2) em 02.03.2026</t>
         </is>
       </c>
       <c r="C1613" s="3" t="n">
-        <v>-82.64</v>
+        <v>-540.29</v>
       </c>
       <c r="D1613" t="inlineStr">
         <is>
-          <t>Serviços Funerários</t>
+          <t>VIAGENS/Passagens</t>
         </is>
       </c>
       <c r="E1613" t="inlineStr">
         <is>
-          <t>Conta BB</t>
+          <t>Cartão BB VISA</t>
         </is>
       </c>
       <c r="F1613" t="inlineStr">
@@ -72053,12 +72048,17 @@
       </c>
       <c r="G1613" t="inlineStr">
         <is>
-          <t>SEGUROS E SERVIÇOS FUNERÁRIOS</t>
+          <t>LAZER</t>
+        </is>
+      </c>
+      <c r="H1613" t="inlineStr">
+        <is>
+          <t>VIAGENS</t>
         </is>
       </c>
       <c r="I1613" t="inlineStr">
         <is>
-          <t>Despesas com Seguros</t>
+          <t>Despesas com lazer</t>
         </is>
       </c>
       <c r="J1613" t="inlineStr">
@@ -72073,15 +72073,15 @@
       </c>
       <c r="B1614" t="inlineStr">
         <is>
-          <t>Presentes comprados por Gracinha (2026.10.14)</t>
+          <t>Hotel Stela Maris - Salvador</t>
         </is>
       </c>
       <c r="C1614" s="3" t="n">
-        <v>-134.38</v>
+        <v>-69.37</v>
       </c>
       <c r="D1614" t="inlineStr">
         <is>
-          <t>Presentes</t>
+          <t>VIAGENS/Estadia</t>
         </is>
       </c>
       <c r="E1614" t="inlineStr">
@@ -72096,12 +72096,17 @@
       </c>
       <c r="G1614" t="inlineStr">
         <is>
-          <t>FAMÍLIA</t>
+          <t>LAZER</t>
+        </is>
+      </c>
+      <c r="H1614" t="inlineStr">
+        <is>
+          <t>VIAGENS</t>
         </is>
       </c>
       <c r="I1614" t="inlineStr">
         <is>
-          <t>Despesas com família</t>
+          <t>Despesas com lazer</t>
         </is>
       </c>
       <c r="J1614" t="inlineStr">
@@ -72116,15 +72121,15 @@
       </c>
       <c r="B1615" t="inlineStr">
         <is>
-          <t>Aplicação PGBL BRASILPREV - ACMD</t>
+          <t>Mensalidade da hidroginástica (11 / 11)</t>
         </is>
       </c>
       <c r="C1615" s="3" t="n">
-        <v>-209.34</v>
+        <v>-23.46</v>
       </c>
       <c r="D1615" t="inlineStr">
         <is>
-          <t>BRASILPREV</t>
+          <t>Academia</t>
         </is>
       </c>
       <c r="E1615" t="inlineStr">
@@ -72139,17 +72144,17 @@
       </c>
       <c r="G1615" t="inlineStr">
         <is>
-          <t>INVESTIMENTOS E PATRIMÔNIO</t>
+          <t>FAMÍLIA</t>
         </is>
       </c>
       <c r="I1615" t="inlineStr">
         <is>
-          <t>Investimentos Financeiros</t>
+          <t>Despesas com família</t>
         </is>
       </c>
       <c r="J1615" t="inlineStr">
         <is>
-          <t>Investimentos Financeiros</t>
+          <t>Despesas e Custos</t>
         </is>
       </c>
     </row>
@@ -72159,15 +72164,15 @@
       </c>
       <c r="B1616" t="inlineStr">
         <is>
-          <t>Hotel Stela Maris - Salvador</t>
+          <t>Aplicação PGBL BRASILPREV - ACMD</t>
         </is>
       </c>
       <c r="C1616" s="3" t="n">
-        <v>-69.37</v>
+        <v>-209.34</v>
       </c>
       <c r="D1616" t="inlineStr">
         <is>
-          <t>VIAGENS/Estadia</t>
+          <t>BRASILPREV</t>
         </is>
       </c>
       <c r="E1616" t="inlineStr">
@@ -72182,45 +72187,40 @@
       </c>
       <c r="G1616" t="inlineStr">
         <is>
-          <t>LAZER</t>
-        </is>
-      </c>
-      <c r="H1616" t="inlineStr">
-        <is>
-          <t>VIAGENS</t>
+          <t>INVESTIMENTOS E PATRIMÔNIO</t>
         </is>
       </c>
       <c r="I1616" t="inlineStr">
         <is>
-          <t>Despesas com lazer</t>
+          <t>Investimentos Financeiros</t>
         </is>
       </c>
       <c r="J1616" t="inlineStr">
         <is>
-          <t>Despesas e Custos</t>
+          <t>Investimentos Financeiros</t>
         </is>
       </c>
     </row>
     <row r="1617">
       <c r="A1617" s="2" t="n">
-        <v>46367</v>
+        <v>46366</v>
       </c>
       <c r="B1617" t="inlineStr">
         <is>
-          <t>Casa Aracaju - Toldo de proteção para a garagem</t>
+          <t>Presentes comprados por Gracinha (2026.10.14)</t>
         </is>
       </c>
       <c r="C1617" s="3" t="n">
-        <v>-1818.04</v>
+        <v>-134.38</v>
       </c>
       <c r="D1617" t="inlineStr">
         <is>
-          <t>Ampliação-Melhorias Imóveis</t>
+          <t>Presentes</t>
         </is>
       </c>
       <c r="E1617" t="inlineStr">
         <is>
-          <t>Cartão BB VISA</t>
+          <t>Conta BB</t>
         </is>
       </c>
       <c r="F1617" t="inlineStr">
@@ -72230,40 +72230,40 @@
       </c>
       <c r="G1617" t="inlineStr">
         <is>
-          <t>BENS DURÁVEIS</t>
+          <t>FAMÍLIA</t>
         </is>
       </c>
       <c r="I1617" t="inlineStr">
         <is>
-          <t>Investimentos Bens Imóveis</t>
+          <t>Despesas com família</t>
         </is>
       </c>
       <c r="J1617" t="inlineStr">
         <is>
-          <t>Investimentos Bens Imóveis</t>
+          <t>Despesas e Custos</t>
         </is>
       </c>
     </row>
     <row r="1618">
       <c r="A1618" s="2" t="n">
-        <v>46369</v>
+        <v>46366</v>
       </c>
       <c r="B1618" t="inlineStr">
         <is>
-          <t>Ajuste Seguro HILUX SW4 para a RANGER XLT</t>
+          <t>Plano OSAF - Serviços Funerários</t>
         </is>
       </c>
       <c r="C1618" s="3" t="n">
-        <v>-93.89</v>
+        <v>-82.64</v>
       </c>
       <c r="D1618" t="inlineStr">
         <is>
-          <t>Automóvel/Seguro</t>
+          <t>Serviços Funerários</t>
         </is>
       </c>
       <c r="E1618" t="inlineStr">
         <is>
-          <t>Cartão BB VISA</t>
+          <t>Conta BB</t>
         </is>
       </c>
       <c r="F1618" t="inlineStr">
@@ -72273,17 +72273,12 @@
       </c>
       <c r="G1618" t="inlineStr">
         <is>
-          <t>TRANSPORTE</t>
-        </is>
-      </c>
-      <c r="H1618" t="inlineStr">
-        <is>
-          <t>Automóvel</t>
+          <t>SEGUROS E SERVIÇOS FUNERÁRIOS</t>
         </is>
       </c>
       <c r="I1618" t="inlineStr">
         <is>
-          <t>Despesas com Automóvel (Seguros)</t>
+          <t>Despesas com Seguros</t>
         </is>
       </c>
       <c r="J1618" t="inlineStr">
@@ -72294,19 +72289,19 @@
     </row>
     <row r="1619">
       <c r="A1619" s="2" t="n">
-        <v>46369</v>
+        <v>46367</v>
       </c>
       <c r="B1619" t="inlineStr">
         <is>
-          <t>Seguro da Hilux SW4</t>
+          <t>Casa Aracaju - Toldo de proteção para a garagem</t>
         </is>
       </c>
       <c r="C1619" s="3" t="n">
-        <v>-233.11</v>
+        <v>-1818.04</v>
       </c>
       <c r="D1619" t="inlineStr">
         <is>
-          <t>Automóvel/Seguro</t>
+          <t>Ampliação-Melhorias Imóveis</t>
         </is>
       </c>
       <c r="E1619" t="inlineStr">
@@ -72321,22 +72316,17 @@
       </c>
       <c r="G1619" t="inlineStr">
         <is>
-          <t>TRANSPORTE</t>
-        </is>
-      </c>
-      <c r="H1619" t="inlineStr">
-        <is>
-          <t>Automóvel</t>
+          <t>BENS DURÁVEIS</t>
         </is>
       </c>
       <c r="I1619" t="inlineStr">
         <is>
-          <t>Despesas com Automóvel (Seguros)</t>
+          <t>Investimentos Bens Imóveis</t>
         </is>
       </c>
       <c r="J1619" t="inlineStr">
         <is>
-          <t>Despesas e Custos</t>
+          <t>Investimentos Bens Imóveis</t>
         </is>
       </c>
     </row>
@@ -72346,15 +72336,15 @@
       </c>
       <c r="B1620" t="inlineStr">
         <is>
-          <t>Casa Aracaju - Cabo PP para interligar o carregador de Bateria do BYD</t>
+          <t>Ajuste Seguro HILUX SW4 para a RANGER XLT</t>
         </is>
       </c>
       <c r="C1620" s="3" t="n">
-        <v>-58.07</v>
+        <v>-93.89</v>
       </c>
       <c r="D1620" t="inlineStr">
         <is>
-          <t>Eletrônicos</t>
+          <t>Automóvel/Seguro</t>
         </is>
       </c>
       <c r="E1620" t="inlineStr">
@@ -72369,35 +72359,40 @@
       </c>
       <c r="G1620" t="inlineStr">
         <is>
-          <t>BENS DURÁVEIS</t>
+          <t>TRANSPORTE</t>
+        </is>
+      </c>
+      <c r="H1620" t="inlineStr">
+        <is>
+          <t>Automóvel</t>
         </is>
       </c>
       <c r="I1620" t="inlineStr">
         <is>
-          <t>Investimentos Bens</t>
+          <t>Despesas com Automóvel (Seguros)</t>
         </is>
       </c>
       <c r="J1620" t="inlineStr">
         <is>
-          <t>Investimentos</t>
+          <t>Despesas e Custos</t>
         </is>
       </c>
     </row>
     <row r="1621">
       <c r="A1621" s="2" t="n">
-        <v>46371</v>
+        <v>46369</v>
       </c>
       <c r="B1621" t="inlineStr">
         <is>
-          <t>Pagamento Clube SMILES</t>
+          <t>Seguro da Hilux SW4</t>
         </is>
       </c>
       <c r="C1621" s="3" t="n">
-        <v>-46</v>
+        <v>-233.11</v>
       </c>
       <c r="D1621" t="inlineStr">
         <is>
-          <t>VIAGENS/Passagens</t>
+          <t>Automóvel/Seguro</t>
         </is>
       </c>
       <c r="E1621" t="inlineStr">
@@ -72412,17 +72407,17 @@
       </c>
       <c r="G1621" t="inlineStr">
         <is>
-          <t>LAZER</t>
+          <t>TRANSPORTE</t>
         </is>
       </c>
       <c r="H1621" t="inlineStr">
         <is>
-          <t>VIAGENS</t>
+          <t>Automóvel</t>
         </is>
       </c>
       <c r="I1621" t="inlineStr">
         <is>
-          <t>Despesas com lazer</t>
+          <t>Despesas com Automóvel (Seguros)</t>
         </is>
       </c>
       <c r="J1621" t="inlineStr">
@@ -72433,19 +72428,19 @@
     </row>
     <row r="1622">
       <c r="A1622" s="2" t="n">
-        <v>46371</v>
+        <v>46369</v>
       </c>
       <c r="B1622" t="inlineStr">
         <is>
-          <t>Remédios para ACMD</t>
+          <t>Casa Aracaju - Cabo PP para interligar o carregador de Bateria do BYD</t>
         </is>
       </c>
       <c r="C1622" s="3" t="n">
-        <v>-52.83</v>
+        <v>-58.07</v>
       </c>
       <c r="D1622" t="inlineStr">
         <is>
-          <t>Farmácia</t>
+          <t>Eletrônicos</t>
         </is>
       </c>
       <c r="E1622" t="inlineStr">
@@ -72460,35 +72455,35 @@
       </c>
       <c r="G1622" t="inlineStr">
         <is>
-          <t>SAÚDE</t>
+          <t>BENS DURÁVEIS</t>
         </is>
       </c>
       <c r="I1622" t="inlineStr">
         <is>
-          <t>Despesas com Saúde</t>
+          <t>Investimentos Bens</t>
         </is>
       </c>
       <c r="J1622" t="inlineStr">
         <is>
-          <t>Despesas e Custos</t>
+          <t>Investimentos</t>
         </is>
       </c>
     </row>
     <row r="1623">
       <c r="A1623" s="2" t="n">
-        <v>46372</v>
+        <v>46371</v>
       </c>
       <c r="B1623" t="inlineStr">
         <is>
-          <t>Transporte Terrestre, Hoteis e Excursão</t>
+          <t>Remédios para ACMD</t>
         </is>
       </c>
       <c r="C1623" s="3" t="n">
-        <v>-1824.26</v>
+        <v>-52.83</v>
       </c>
       <c r="D1623" t="inlineStr">
         <is>
-          <t>VIAGENS/Passeios</t>
+          <t>Farmácia</t>
         </is>
       </c>
       <c r="E1623" t="inlineStr">
@@ -72503,17 +72498,12 @@
       </c>
       <c r="G1623" t="inlineStr">
         <is>
-          <t>LAZER</t>
-        </is>
-      </c>
-      <c r="H1623" t="inlineStr">
-        <is>
-          <t>VIAGENS</t>
+          <t>SAÚDE</t>
         </is>
       </c>
       <c r="I1623" t="inlineStr">
         <is>
-          <t>Despesas com lazer</t>
+          <t>Despesas com Saúde</t>
         </is>
       </c>
       <c r="J1623" t="inlineStr">
@@ -72524,19 +72514,19 @@
     </row>
     <row r="1624">
       <c r="A1624" s="2" t="n">
-        <v>46375</v>
+        <v>46371</v>
       </c>
       <c r="B1624" t="inlineStr">
         <is>
-          <t>Perfume no Boticário</t>
+          <t>Pagamento Clube SMILES</t>
         </is>
       </c>
       <c r="C1624" s="3" t="n">
-        <v>-8.99</v>
+        <v>-46</v>
       </c>
       <c r="D1624" t="inlineStr">
         <is>
-          <t>Salão de Beleza e Cosméticos</t>
+          <t>VIAGENS/Passagens</t>
         </is>
       </c>
       <c r="E1624" t="inlineStr">
@@ -72551,12 +72541,17 @@
       </c>
       <c r="G1624" t="inlineStr">
         <is>
-          <t>FAMÍLIA</t>
+          <t>LAZER</t>
+        </is>
+      </c>
+      <c r="H1624" t="inlineStr">
+        <is>
+          <t>VIAGENS</t>
         </is>
       </c>
       <c r="I1624" t="inlineStr">
         <is>
-          <t>Despesas com família</t>
+          <t>Despesas com lazer</t>
         </is>
       </c>
       <c r="J1624" t="inlineStr">
@@ -72567,19 +72562,19 @@
     </row>
     <row r="1625">
       <c r="A1625" s="2" t="n">
-        <v>46378</v>
+        <v>46372</v>
       </c>
       <c r="B1625" t="inlineStr">
         <is>
-          <t>Lata de lixo e outros utensílios domésticos</t>
+          <t>Transporte Terrestre, Hoteis e Excursão</t>
         </is>
       </c>
       <c r="C1625" s="3" t="n">
-        <v>-53.66</v>
+        <v>-1824.26</v>
       </c>
       <c r="D1625" t="inlineStr">
         <is>
-          <t>Restauração e Manutenção</t>
+          <t>VIAGENS/Passeios</t>
         </is>
       </c>
       <c r="E1625" t="inlineStr">
@@ -72594,17 +72589,17 @@
       </c>
       <c r="G1625" t="inlineStr">
         <is>
-          <t>IMÓVEIS</t>
+          <t>LAZER</t>
         </is>
       </c>
       <c r="H1625" t="inlineStr">
         <is>
-          <t>Manutenção e encargos</t>
+          <t>VIAGENS</t>
         </is>
       </c>
       <c r="I1625" t="inlineStr">
         <is>
-          <t>Despesas com imóveis</t>
+          <t>Despesas com lazer</t>
         </is>
       </c>
       <c r="J1625" t="inlineStr">
@@ -72615,19 +72610,19 @@
     </row>
     <row r="1626">
       <c r="A1626" s="2" t="n">
-        <v>46378</v>
+        <v>46375</v>
       </c>
       <c r="B1626" t="inlineStr">
         <is>
-          <t>Casa Aracaju - Materiais para o jardim</t>
+          <t>Perfume no Boticário</t>
         </is>
       </c>
       <c r="C1626" s="3" t="n">
-        <v>-112.07</v>
+        <v>-8.99</v>
       </c>
       <c r="D1626" t="inlineStr">
         <is>
-          <t>Restauração e Manutenção</t>
+          <t>Salão de Beleza e Cosméticos</t>
         </is>
       </c>
       <c r="E1626" t="inlineStr">
@@ -72642,17 +72637,12 @@
       </c>
       <c r="G1626" t="inlineStr">
         <is>
-          <t>IMÓVEIS</t>
-        </is>
-      </c>
-      <c r="H1626" t="inlineStr">
-        <is>
-          <t>Manutenção e encargos</t>
+          <t>FAMÍLIA</t>
         </is>
       </c>
       <c r="I1626" t="inlineStr">
         <is>
-          <t>Despesas com imóveis</t>
+          <t>Despesas com família</t>
         </is>
       </c>
       <c r="J1626" t="inlineStr">
@@ -72663,19 +72653,19 @@
     </row>
     <row r="1627">
       <c r="A1627" s="2" t="n">
-        <v>46380</v>
+        <v>46378</v>
       </c>
       <c r="B1627" t="inlineStr">
         <is>
-          <t>Instalação das câmeras lateral e frontal na RANGER xLT</t>
+          <t>Lata de lixo e outros utensílios domésticos</t>
         </is>
       </c>
       <c r="C1627" s="3" t="n">
-        <v>-500</v>
+        <v>-53.66</v>
       </c>
       <c r="D1627" t="inlineStr">
         <is>
-          <t>Automóvel/Manutenção</t>
+          <t>Restauração e Manutenção</t>
         </is>
       </c>
       <c r="E1627" t="inlineStr">
@@ -72690,17 +72680,17 @@
       </c>
       <c r="G1627" t="inlineStr">
         <is>
-          <t>TRANSPORTE</t>
+          <t>IMÓVEIS</t>
         </is>
       </c>
       <c r="H1627" t="inlineStr">
         <is>
-          <t>Automóvel</t>
+          <t>Manutenção e encargos</t>
         </is>
       </c>
       <c r="I1627" t="inlineStr">
         <is>
-          <t>Despesas com Automóvel (Manutenção)</t>
+          <t>Despesas com imóveis</t>
         </is>
       </c>
       <c r="J1627" t="inlineStr">
@@ -72711,19 +72701,19 @@
     </row>
     <row r="1628">
       <c r="A1628" s="2" t="n">
-        <v>46383</v>
+        <v>46378</v>
       </c>
       <c r="B1628" t="inlineStr">
         <is>
-          <t>Troca da bateria do MACBOOK PRO</t>
+          <t>Casa Aracaju - Materiais para o jardim</t>
         </is>
       </c>
       <c r="C1628" s="3" t="n">
-        <v>-102.5</v>
+        <v>-112.07</v>
       </c>
       <c r="D1628" t="inlineStr">
         <is>
-          <t>OUTRAS DESPESAS</t>
+          <t>Restauração e Manutenção</t>
         </is>
       </c>
       <c r="E1628" t="inlineStr">
@@ -72738,12 +72728,17 @@
       </c>
       <c r="G1628" t="inlineStr">
         <is>
-          <t>OUTRAS DESPESAS</t>
+          <t>IMÓVEIS</t>
+        </is>
+      </c>
+      <c r="H1628" t="inlineStr">
+        <is>
+          <t>Manutenção e encargos</t>
         </is>
       </c>
       <c r="I1628" t="inlineStr">
         <is>
-          <t>Outras Despesas</t>
+          <t>Despesas com imóveis</t>
         </is>
       </c>
       <c r="J1628" t="inlineStr">
@@ -72754,19 +72749,19 @@
     </row>
     <row r="1629">
       <c r="A1629" s="2" t="n">
-        <v>46383</v>
+        <v>46380</v>
       </c>
       <c r="B1629" t="inlineStr">
         <is>
-          <t>Aquisição do celular MOTOROLA G86</t>
+          <t>Instalação das câmeras lateral e frontal na RANGER xLT</t>
         </is>
       </c>
       <c r="C1629" s="3" t="n">
-        <v>-139</v>
+        <v>-500</v>
       </c>
       <c r="D1629" t="inlineStr">
         <is>
-          <t>Eletrônicos</t>
+          <t>Automóvel/Manutenção</t>
         </is>
       </c>
       <c r="E1629" t="inlineStr">
@@ -72781,65 +72776,156 @@
       </c>
       <c r="G1629" t="inlineStr">
         <is>
-          <t>BENS DURÁVEIS</t>
+          <t>TRANSPORTE</t>
+        </is>
+      </c>
+      <c r="H1629" t="inlineStr">
+        <is>
+          <t>Automóvel</t>
         </is>
       </c>
       <c r="I1629" t="inlineStr">
         <is>
-          <t>Investimentos Bens</t>
+          <t>Despesas com Automóvel (Manutenção)</t>
         </is>
       </c>
       <c r="J1629" t="inlineStr">
         <is>
-          <t>Investimentos</t>
+          <t>Despesas e Custos</t>
         </is>
       </c>
     </row>
     <row r="1630">
       <c r="A1630" s="2" t="n">
+        <v>46383</v>
+      </c>
+      <c r="B1630" t="inlineStr">
+        <is>
+          <t>Troca da bateria do MACBOOK PRO</t>
+        </is>
+      </c>
+      <c r="C1630" s="3" t="n">
+        <v>-102.5</v>
+      </c>
+      <c r="D1630" t="inlineStr">
+        <is>
+          <t>OUTRAS DESPESAS</t>
+        </is>
+      </c>
+      <c r="E1630" t="inlineStr">
+        <is>
+          <t>Cartão BB VISA</t>
+        </is>
+      </c>
+      <c r="F1630" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
+      <c r="G1630" t="inlineStr">
+        <is>
+          <t>OUTRAS DESPESAS</t>
+        </is>
+      </c>
+      <c r="I1630" t="inlineStr">
+        <is>
+          <t>Outras Despesas</t>
+        </is>
+      </c>
+      <c r="J1630" t="inlineStr">
+        <is>
+          <t>Despesas e Custos</t>
+        </is>
+      </c>
+    </row>
+    <row r="1631">
+      <c r="A1631" s="2" t="n">
+        <v>46383</v>
+      </c>
+      <c r="B1631" t="inlineStr">
+        <is>
+          <t>Aquisição do celular MOTOROLA G86</t>
+        </is>
+      </c>
+      <c r="C1631" s="3" t="n">
+        <v>-139</v>
+      </c>
+      <c r="D1631" t="inlineStr">
+        <is>
+          <t>Eletrônicos</t>
+        </is>
+      </c>
+      <c r="E1631" t="inlineStr">
+        <is>
+          <t>Cartão BB VISA</t>
+        </is>
+      </c>
+      <c r="F1631" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
+      <c r="G1631" t="inlineStr">
+        <is>
+          <t>BENS DURÁVEIS</t>
+        </is>
+      </c>
+      <c r="I1631" t="inlineStr">
+        <is>
+          <t>Investimentos Bens</t>
+        </is>
+      </c>
+      <c r="J1631" t="inlineStr">
+        <is>
+          <t>Investimentos</t>
+        </is>
+      </c>
+    </row>
+    <row r="1632">
+      <c r="A1632" s="2" t="n">
         <v>46384</v>
       </c>
-      <c r="B1630" t="inlineStr">
+      <c r="B1632" t="inlineStr">
         <is>
           <t>TV SAMSUNG quarto do casal (8 / 8)</t>
         </is>
       </c>
-      <c r="C1630" s="3" t="n">
+      <c r="C1632" s="3" t="n">
         <v>-337.48</v>
       </c>
-      <c r="D1630" t="inlineStr">
+      <c r="D1632" t="inlineStr">
         <is>
           <t>Acessórios</t>
         </is>
       </c>
-      <c r="E1630" t="inlineStr">
-        <is>
-          <t>Cartão BB VISA</t>
-        </is>
-      </c>
-      <c r="F1630" t="inlineStr">
+      <c r="E1632" t="inlineStr">
+        <is>
+          <t>Cartão BB VISA</t>
+        </is>
+      </c>
+      <c r="F1632" t="inlineStr">
         <is>
           <t>Não</t>
         </is>
       </c>
-      <c r="G1630" t="inlineStr">
+      <c r="G1632" t="inlineStr">
         <is>
           <t>FAMÍLIA</t>
         </is>
       </c>
-      <c r="I1630" t="inlineStr">
+      <c r="I1632" t="inlineStr">
         <is>
           <t>Despesas com família</t>
         </is>
       </c>
-      <c r="J1630" t="inlineStr">
+      <c r="J1632" t="inlineStr">
         <is>
           <t>Despesas e Custos</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:J1630"/>
+  <autoFilter ref="A1:J1632"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>